<commit_message>
Clean up documentation and presentation assets
</commit_message>
<xml_diff>
--- a/doc/gantt_bobtricks.xlsx
+++ b/doc/gantt_bobtricks.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -236,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -300,7 +299,7 @@
     <xf numFmtId="0" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -316,7 +315,7 @@
     <xf numFmtId="0" fontId="9" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -331,7 +330,7 @@
     <xf numFmtId="0" fontId="9" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -346,7 +345,7 @@
     <xf numFmtId="0" fontId="9" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -361,7 +360,7 @@
     <xf numFmtId="0" fontId="9" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -381,7 +380,7 @@
     <xf numFmtId="0" fontId="9" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -393,12 +392,33 @@
     <xf numFmtId="0" fontId="9" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -767,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB166"/>
+  <dimension ref="A1:BD175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -824,6 +844,8 @@
     <col width="3.2" customWidth="1" min="52" max="52"/>
     <col width="3.2" customWidth="1" min="53" max="53"/>
     <col width="3.2" customWidth="1" min="54" max="54"/>
+    <col width="3.2" customWidth="1" min="55" max="55"/>
+    <col width="3.2" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -836,7 +858,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Période : 9 mars 2026 – 25 avril 2026   ·   149 tâches   ·   7 phases de développement</t>
+          <t>Période : 9 mars 2026 – 27 avril 2026   ·   157 tâches   ·   8 phases de développement</t>
         </is>
       </c>
     </row>
@@ -887,7 +909,7 @@
       </c>
       <c r="AN5" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Phase 7 — Refactoring et modularisation</t>
+          <t xml:space="preserve">  Phase 7 — Refactoring et modularisation   ·   Phase 8 — Finalisation soutenance</t>
         </is>
       </c>
     </row>
@@ -1175,6 +1197,16 @@
       <c r="BB8" s="16" t="inlineStr">
         <is>
           <t>S</t>
+        </is>
+      </c>
+      <c r="BC8" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="BD8" s="16" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
     </row>
@@ -1322,6 +1354,12 @@
       </c>
       <c r="BB9" s="18" t="n">
         <v>25</v>
+      </c>
+      <c r="BC9" s="18" t="n">
+        <v>26</v>
+      </c>
+      <c r="BD9" s="18" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
@@ -1378,6 +1416,8 @@
       <c r="AZ10" s="20" t="n"/>
       <c r="BA10" s="20" t="n"/>
       <c r="BB10" s="20" t="n"/>
+      <c r="BC10" s="20" t="n"/>
+      <c r="BD10" s="20" t="n"/>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="21" t="n">
@@ -1393,10 +1433,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="72" t="n">
         <v>46093</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="72" t="n">
         <v>46093</v>
       </c>
       <c r="F11" s="21" t="n">
@@ -1454,6 +1494,8 @@
       <c r="AZ11" s="24" t="n"/>
       <c r="BA11" s="24" t="n"/>
       <c r="BB11" s="26" t="n"/>
+      <c r="BC11" s="26" t="n"/>
+      <c r="BD11" s="26" t="n"/>
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="21" t="n">
@@ -1469,10 +1511,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="72" t="n">
         <v>46093</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="72" t="n">
         <v>46093</v>
       </c>
       <c r="F12" s="21" t="n">
@@ -1530,6 +1572,8 @@
       <c r="AZ12" s="24" t="n"/>
       <c r="BA12" s="24" t="n"/>
       <c r="BB12" s="26" t="n"/>
+      <c r="BC12" s="26" t="n"/>
+      <c r="BD12" s="26" t="n"/>
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="21" t="n">
@@ -1545,10 +1589,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="72" t="n">
         <v>46093</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="72" t="n">
         <v>46094</v>
       </c>
       <c r="F13" s="21" t="n">
@@ -1602,6 +1646,8 @@
       <c r="AZ13" s="24" t="n"/>
       <c r="BA13" s="24" t="n"/>
       <c r="BB13" s="26" t="n"/>
+      <c r="BC13" s="26" t="n"/>
+      <c r="BD13" s="26" t="n"/>
     </row>
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="21" t="n">
@@ -1617,10 +1663,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="72" t="n">
         <v>46094</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="72" t="n">
         <v>46094</v>
       </c>
       <c r="F14" s="21" t="n">
@@ -1678,6 +1724,8 @@
       <c r="AZ14" s="24" t="n"/>
       <c r="BA14" s="24" t="n"/>
       <c r="BB14" s="26" t="n"/>
+      <c r="BC14" s="26" t="n"/>
+      <c r="BD14" s="26" t="n"/>
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="21" t="n">
@@ -1693,10 +1741,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="72" t="n">
         <v>46094</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="72" t="n">
         <v>46094</v>
       </c>
       <c r="F15" s="21" t="n">
@@ -1754,6 +1802,8 @@
       <c r="AZ15" s="24" t="n"/>
       <c r="BA15" s="24" t="n"/>
       <c r="BB15" s="26" t="n"/>
+      <c r="BC15" s="26" t="n"/>
+      <c r="BD15" s="26" t="n"/>
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="21" t="n">
@@ -1769,10 +1819,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="72" t="n">
         <v>46094</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F16" s="21" t="n">
@@ -1826,6 +1876,8 @@
       <c r="AZ16" s="24" t="n"/>
       <c r="BA16" s="24" t="n"/>
       <c r="BB16" s="26" t="n"/>
+      <c r="BC16" s="26" t="n"/>
+      <c r="BD16" s="26" t="n"/>
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="21" t="n">
@@ -1841,10 +1893,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="72" t="n">
         <v>46094</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F17" s="21" t="n">
@@ -1898,6 +1950,8 @@
       <c r="AZ17" s="24" t="n"/>
       <c r="BA17" s="24" t="n"/>
       <c r="BB17" s="26" t="n"/>
+      <c r="BC17" s="26" t="n"/>
+      <c r="BD17" s="26" t="n"/>
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="21" t="n">
@@ -1913,10 +1967,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="72" t="n">
         <v>46094</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="72" t="n">
         <v>46094</v>
       </c>
       <c r="F18" s="21" t="n">
@@ -1974,6 +2028,8 @@
       <c r="AZ18" s="24" t="n"/>
       <c r="BA18" s="24" t="n"/>
       <c r="BB18" s="26" t="n"/>
+      <c r="BC18" s="26" t="n"/>
+      <c r="BD18" s="26" t="n"/>
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="21" t="n">
@@ -1989,10 +2045,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="72" t="n">
         <v>46093</v>
       </c>
-      <c r="E19" s="23" t="n">
+      <c r="E19" s="72" t="n">
         <v>46094</v>
       </c>
       <c r="F19" s="21" t="n">
@@ -2046,6 +2102,8 @@
       <c r="AZ19" s="24" t="n"/>
       <c r="BA19" s="24" t="n"/>
       <c r="BB19" s="26" t="n"/>
+      <c r="BC19" s="26" t="n"/>
+      <c r="BD19" s="26" t="n"/>
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="21" t="n">
@@ -2061,10 +2119,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E20" s="23" t="n">
+      <c r="E20" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F20" s="21" t="n">
@@ -2122,6 +2180,8 @@
       <c r="AZ20" s="24" t="n"/>
       <c r="BA20" s="24" t="n"/>
       <c r="BB20" s="26" t="n"/>
+      <c r="BC20" s="26" t="n"/>
+      <c r="BD20" s="26" t="n"/>
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="21" t="n">
@@ -2137,10 +2197,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F21" s="21" t="n">
@@ -2198,6 +2258,8 @@
       <c r="AZ21" s="24" t="n"/>
       <c r="BA21" s="24" t="n"/>
       <c r="BB21" s="26" t="n"/>
+      <c r="BC21" s="26" t="n"/>
+      <c r="BD21" s="26" t="n"/>
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="21" t="n">
@@ -2213,10 +2275,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E22" s="23" t="n">
+      <c r="E22" s="72" t="n">
         <v>46096</v>
       </c>
       <c r="F22" s="21" t="n">
@@ -2270,6 +2332,8 @@
       <c r="AZ22" s="24" t="n"/>
       <c r="BA22" s="24" t="n"/>
       <c r="BB22" s="26" t="n"/>
+      <c r="BC22" s="26" t="n"/>
+      <c r="BD22" s="26" t="n"/>
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="21" t="n">
@@ -2285,10 +2349,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D23" s="23" t="n">
+      <c r="D23" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E23" s="23" t="n">
+      <c r="E23" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F23" s="21" t="n">
@@ -2346,6 +2410,8 @@
       <c r="AZ23" s="24" t="n"/>
       <c r="BA23" s="24" t="n"/>
       <c r="BB23" s="26" t="n"/>
+      <c r="BC23" s="26" t="n"/>
+      <c r="BD23" s="26" t="n"/>
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="21" t="n">
@@ -2361,10 +2427,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D24" s="23" t="n">
+      <c r="D24" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E24" s="23" t="n">
+      <c r="E24" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F24" s="21" t="n">
@@ -2422,6 +2488,8 @@
       <c r="AZ24" s="24" t="n"/>
       <c r="BA24" s="24" t="n"/>
       <c r="BB24" s="26" t="n"/>
+      <c r="BC24" s="26" t="n"/>
+      <c r="BD24" s="26" t="n"/>
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="21" t="n">
@@ -2437,10 +2505,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D25" s="23" t="n">
+      <c r="D25" s="72" t="n">
         <v>46094</v>
       </c>
-      <c r="E25" s="23" t="n">
+      <c r="E25" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F25" s="21" t="n">
@@ -2494,6 +2562,8 @@
       <c r="AZ25" s="24" t="n"/>
       <c r="BA25" s="24" t="n"/>
       <c r="BB25" s="26" t="n"/>
+      <c r="BC25" s="26" t="n"/>
+      <c r="BD25" s="26" t="n"/>
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="21" t="n">
@@ -2509,10 +2579,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D26" s="23" t="n">
+      <c r="D26" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E26" s="23" t="n">
+      <c r="E26" s="72" t="n">
         <v>46095</v>
       </c>
       <c r="F26" s="21" t="n">
@@ -2570,6 +2640,8 @@
       <c r="AZ26" s="24" t="n"/>
       <c r="BA26" s="24" t="n"/>
       <c r="BB26" s="26" t="n"/>
+      <c r="BC26" s="26" t="n"/>
+      <c r="BD26" s="26" t="n"/>
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="21" t="n">
@@ -2585,10 +2657,10 @@
           <t>Ph.0</t>
         </is>
       </c>
-      <c r="D27" s="23" t="n">
+      <c r="D27" s="72" t="n">
         <v>46095</v>
       </c>
-      <c r="E27" s="23" t="n">
+      <c r="E27" s="72" t="n">
         <v>46096</v>
       </c>
       <c r="F27" s="21" t="n">
@@ -2642,6 +2714,8 @@
       <c r="AZ27" s="24" t="n"/>
       <c r="BA27" s="24" t="n"/>
       <c r="BB27" s="26" t="n"/>
+      <c r="BC27" s="26" t="n"/>
+      <c r="BD27" s="26" t="n"/>
     </row>
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -2697,6 +2771,8 @@
       <c r="AZ28" s="28" t="n"/>
       <c r="BA28" s="28" t="n"/>
       <c r="BB28" s="28" t="n"/>
+      <c r="BC28" s="28" t="n"/>
+      <c r="BD28" s="28" t="n"/>
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="29" t="n">
@@ -2712,10 +2788,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D29" s="31" t="n">
+      <c r="D29" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E29" s="31" t="n">
+      <c r="E29" s="73" t="n">
         <v>46101</v>
       </c>
       <c r="F29" s="29" t="n">
@@ -2773,6 +2849,8 @@
       <c r="AZ29" s="32" t="n"/>
       <c r="BA29" s="32" t="n"/>
       <c r="BB29" s="26" t="n"/>
+      <c r="BC29" s="26" t="n"/>
+      <c r="BD29" s="26" t="n"/>
     </row>
     <row r="30" ht="13" customHeight="1">
       <c r="A30" s="29" t="n">
@@ -2788,10 +2866,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D30" s="31" t="n">
+      <c r="D30" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E30" s="31" t="n">
+      <c r="E30" s="73" t="n">
         <v>46101</v>
       </c>
       <c r="F30" s="29" t="n">
@@ -2849,6 +2927,8 @@
       <c r="AZ30" s="32" t="n"/>
       <c r="BA30" s="32" t="n"/>
       <c r="BB30" s="26" t="n"/>
+      <c r="BC30" s="26" t="n"/>
+      <c r="BD30" s="26" t="n"/>
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" s="29" t="n">
@@ -2864,10 +2944,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D31" s="31" t="n">
+      <c r="D31" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E31" s="31" t="n">
+      <c r="E31" s="73" t="n">
         <v>46102</v>
       </c>
       <c r="F31" s="29" t="n">
@@ -2921,6 +3001,8 @@
       <c r="AZ31" s="32" t="n"/>
       <c r="BA31" s="32" t="n"/>
       <c r="BB31" s="26" t="n"/>
+      <c r="BC31" s="26" t="n"/>
+      <c r="BD31" s="26" t="n"/>
     </row>
     <row r="32" ht="13" customHeight="1">
       <c r="A32" s="29" t="n">
@@ -2936,10 +3018,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D32" s="31" t="n">
+      <c r="D32" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E32" s="31" t="n">
+      <c r="E32" s="73" t="n">
         <v>46101</v>
       </c>
       <c r="F32" s="29" t="n">
@@ -2997,6 +3079,8 @@
       <c r="AZ32" s="32" t="n"/>
       <c r="BA32" s="32" t="n"/>
       <c r="BB32" s="26" t="n"/>
+      <c r="BC32" s="26" t="n"/>
+      <c r="BD32" s="26" t="n"/>
     </row>
     <row r="33" ht="13" customHeight="1">
       <c r="A33" s="29" t="n">
@@ -3012,10 +3096,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D33" s="31" t="n">
+      <c r="D33" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E33" s="31" t="n">
+      <c r="E33" s="73" t="n">
         <v>46101</v>
       </c>
       <c r="F33" s="29" t="n">
@@ -3073,6 +3157,8 @@
       <c r="AZ33" s="32" t="n"/>
       <c r="BA33" s="32" t="n"/>
       <c r="BB33" s="26" t="n"/>
+      <c r="BC33" s="26" t="n"/>
+      <c r="BD33" s="26" t="n"/>
     </row>
     <row r="34" ht="13" customHeight="1">
       <c r="A34" s="29" t="n">
@@ -3088,10 +3174,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D34" s="31" t="n">
+      <c r="D34" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E34" s="31" t="n">
+      <c r="E34" s="73" t="n">
         <v>46102</v>
       </c>
       <c r="F34" s="29" t="n">
@@ -3145,6 +3231,8 @@
       <c r="AZ34" s="32" t="n"/>
       <c r="BA34" s="32" t="n"/>
       <c r="BB34" s="26" t="n"/>
+      <c r="BC34" s="26" t="n"/>
+      <c r="BD34" s="26" t="n"/>
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="29" t="n">
@@ -3160,10 +3248,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D35" s="31" t="n">
+      <c r="D35" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E35" s="31" t="n">
+      <c r="E35" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F35" s="29" t="n">
@@ -3217,6 +3305,8 @@
       <c r="AZ35" s="32" t="n"/>
       <c r="BA35" s="32" t="n"/>
       <c r="BB35" s="26" t="n"/>
+      <c r="BC35" s="26" t="n"/>
+      <c r="BD35" s="26" t="n"/>
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" s="29" t="n">
@@ -3232,10 +3322,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D36" s="31" t="n">
+      <c r="D36" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E36" s="31" t="n">
+      <c r="E36" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F36" s="29" t="n">
@@ -3289,6 +3379,8 @@
       <c r="AZ36" s="32" t="n"/>
       <c r="BA36" s="32" t="n"/>
       <c r="BB36" s="26" t="n"/>
+      <c r="BC36" s="26" t="n"/>
+      <c r="BD36" s="26" t="n"/>
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="29" t="n">
@@ -3304,10 +3396,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D37" s="31" t="n">
+      <c r="D37" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E37" s="31" t="n">
+      <c r="E37" s="73" t="n">
         <v>46102</v>
       </c>
       <c r="F37" s="29" t="n">
@@ -3361,6 +3453,8 @@
       <c r="AZ37" s="32" t="n"/>
       <c r="BA37" s="32" t="n"/>
       <c r="BB37" s="26" t="n"/>
+      <c r="BC37" s="26" t="n"/>
+      <c r="BD37" s="26" t="n"/>
     </row>
     <row r="38" ht="13" customHeight="1">
       <c r="A38" s="29" t="n">
@@ -3376,10 +3470,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D38" s="31" t="n">
+      <c r="D38" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E38" s="31" t="n">
+      <c r="E38" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F38" s="29" t="n">
@@ -3433,6 +3527,8 @@
       <c r="AZ38" s="32" t="n"/>
       <c r="BA38" s="32" t="n"/>
       <c r="BB38" s="26" t="n"/>
+      <c r="BC38" s="26" t="n"/>
+      <c r="BD38" s="26" t="n"/>
     </row>
     <row r="39" ht="13" customHeight="1">
       <c r="A39" s="29" t="n">
@@ -3448,10 +3544,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D39" s="31" t="n">
+      <c r="D39" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E39" s="31" t="n">
+      <c r="E39" s="73" t="n">
         <v>46102</v>
       </c>
       <c r="F39" s="29" t="n">
@@ -3509,6 +3605,8 @@
       <c r="AZ39" s="32" t="n"/>
       <c r="BA39" s="32" t="n"/>
       <c r="BB39" s="26" t="n"/>
+      <c r="BC39" s="26" t="n"/>
+      <c r="BD39" s="26" t="n"/>
     </row>
     <row r="40" ht="13" customHeight="1">
       <c r="A40" s="29" t="n">
@@ -3524,10 +3622,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D40" s="31" t="n">
+      <c r="D40" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E40" s="31" t="n">
+      <c r="E40" s="73" t="n">
         <v>46102</v>
       </c>
       <c r="F40" s="29" t="n">
@@ -3585,6 +3683,8 @@
       <c r="AZ40" s="32" t="n"/>
       <c r="BA40" s="32" t="n"/>
       <c r="BB40" s="26" t="n"/>
+      <c r="BC40" s="26" t="n"/>
+      <c r="BD40" s="26" t="n"/>
     </row>
     <row r="41" ht="13" customHeight="1">
       <c r="A41" s="29" t="n">
@@ -3600,10 +3700,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D41" s="31" t="n">
+      <c r="D41" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E41" s="31" t="n">
+      <c r="E41" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F41" s="29" t="n">
@@ -3657,6 +3757,8 @@
       <c r="AZ41" s="32" t="n"/>
       <c r="BA41" s="32" t="n"/>
       <c r="BB41" s="26" t="n"/>
+      <c r="BC41" s="26" t="n"/>
+      <c r="BD41" s="26" t="n"/>
     </row>
     <row r="42" ht="13" customHeight="1">
       <c r="A42" s="29" t="n">
@@ -3672,10 +3774,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D42" s="31" t="n">
+      <c r="D42" s="73" t="n">
         <v>46101</v>
       </c>
-      <c r="E42" s="31" t="n">
+      <c r="E42" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F42" s="29" t="n">
@@ -3729,6 +3831,8 @@
       <c r="AZ42" s="32" t="n"/>
       <c r="BA42" s="32" t="n"/>
       <c r="BB42" s="26" t="n"/>
+      <c r="BC42" s="26" t="n"/>
+      <c r="BD42" s="26" t="n"/>
     </row>
     <row r="43" ht="13" customHeight="1">
       <c r="A43" s="29" t="n">
@@ -3744,10 +3848,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D43" s="31" t="n">
+      <c r="D43" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E43" s="31" t="n">
+      <c r="E43" s="73" t="n">
         <v>46102</v>
       </c>
       <c r="F43" s="29" t="n">
@@ -3805,6 +3909,8 @@
       <c r="AZ43" s="32" t="n"/>
       <c r="BA43" s="32" t="n"/>
       <c r="BB43" s="26" t="n"/>
+      <c r="BC43" s="26" t="n"/>
+      <c r="BD43" s="26" t="n"/>
     </row>
     <row r="44" ht="13" customHeight="1">
       <c r="A44" s="29" t="n">
@@ -3820,10 +3926,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D44" s="31" t="n">
+      <c r="D44" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E44" s="31" t="n">
+      <c r="E44" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F44" s="29" t="n">
@@ -3877,6 +3983,8 @@
       <c r="AZ44" s="32" t="n"/>
       <c r="BA44" s="32" t="n"/>
       <c r="BB44" s="26" t="n"/>
+      <c r="BC44" s="26" t="n"/>
+      <c r="BD44" s="26" t="n"/>
     </row>
     <row r="45" ht="13" customHeight="1">
       <c r="A45" s="29" t="n">
@@ -3892,10 +4000,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D45" s="31" t="n">
+      <c r="D45" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E45" s="31" t="n">
+      <c r="E45" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F45" s="29" t="n">
@@ -3949,6 +4057,8 @@
       <c r="AZ45" s="32" t="n"/>
       <c r="BA45" s="32" t="n"/>
       <c r="BB45" s="26" t="n"/>
+      <c r="BC45" s="26" t="n"/>
+      <c r="BD45" s="26" t="n"/>
     </row>
     <row r="46" ht="13" customHeight="1">
       <c r="A46" s="29" t="n">
@@ -3964,10 +4074,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D46" s="31" t="n">
+      <c r="D46" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E46" s="31" t="n">
+      <c r="E46" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F46" s="29" t="n">
@@ -4025,6 +4135,8 @@
       <c r="AZ46" s="32" t="n"/>
       <c r="BA46" s="32" t="n"/>
       <c r="BB46" s="26" t="n"/>
+      <c r="BC46" s="26" t="n"/>
+      <c r="BD46" s="26" t="n"/>
     </row>
     <row r="47" ht="13" customHeight="1">
       <c r="A47" s="29" t="n">
@@ -4040,10 +4152,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D47" s="31" t="n">
+      <c r="D47" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E47" s="31" t="n">
+      <c r="E47" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F47" s="29" t="n">
@@ -4097,6 +4209,8 @@
       <c r="AZ47" s="32" t="n"/>
       <c r="BA47" s="32" t="n"/>
       <c r="BB47" s="26" t="n"/>
+      <c r="BC47" s="26" t="n"/>
+      <c r="BD47" s="26" t="n"/>
     </row>
     <row r="48" ht="13" customHeight="1">
       <c r="A48" s="29" t="n">
@@ -4112,10 +4226,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D48" s="31" t="n">
+      <c r="D48" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E48" s="31" t="n">
+      <c r="E48" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F48" s="29" t="n">
@@ -4173,6 +4287,8 @@
       <c r="AZ48" s="32" t="n"/>
       <c r="BA48" s="32" t="n"/>
       <c r="BB48" s="26" t="n"/>
+      <c r="BC48" s="26" t="n"/>
+      <c r="BD48" s="26" t="n"/>
     </row>
     <row r="49" ht="13" customHeight="1">
       <c r="A49" s="29" t="n">
@@ -4188,10 +4304,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D49" s="31" t="n">
+      <c r="D49" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E49" s="31" t="n">
+      <c r="E49" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F49" s="29" t="n">
@@ -4245,6 +4361,8 @@
       <c r="AZ49" s="32" t="n"/>
       <c r="BA49" s="32" t="n"/>
       <c r="BB49" s="26" t="n"/>
+      <c r="BC49" s="26" t="n"/>
+      <c r="BD49" s="26" t="n"/>
     </row>
     <row r="50" ht="13" customHeight="1">
       <c r="A50" s="29" t="n">
@@ -4260,10 +4378,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D50" s="31" t="n">
+      <c r="D50" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E50" s="31" t="n">
+      <c r="E50" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F50" s="29" t="n">
@@ -4317,6 +4435,8 @@
       <c r="AZ50" s="32" t="n"/>
       <c r="BA50" s="32" t="n"/>
       <c r="BB50" s="26" t="n"/>
+      <c r="BC50" s="26" t="n"/>
+      <c r="BD50" s="26" t="n"/>
     </row>
     <row r="51" ht="13" customHeight="1">
       <c r="A51" s="29" t="n">
@@ -4332,10 +4452,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D51" s="31" t="n">
+      <c r="D51" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E51" s="31" t="n">
+      <c r="E51" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F51" s="29" t="n">
@@ -4393,6 +4513,8 @@
       <c r="AZ51" s="32" t="n"/>
       <c r="BA51" s="32" t="n"/>
       <c r="BB51" s="26" t="n"/>
+      <c r="BC51" s="26" t="n"/>
+      <c r="BD51" s="26" t="n"/>
     </row>
     <row r="52" ht="13" customHeight="1">
       <c r="A52" s="29" t="n">
@@ -4408,10 +4530,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D52" s="31" t="n">
+      <c r="D52" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E52" s="31" t="n">
+      <c r="E52" s="73" t="n">
         <v>46105</v>
       </c>
       <c r="F52" s="29" t="n">
@@ -4465,6 +4587,8 @@
       <c r="AZ52" s="32" t="n"/>
       <c r="BA52" s="32" t="n"/>
       <c r="BB52" s="26" t="n"/>
+      <c r="BC52" s="26" t="n"/>
+      <c r="BD52" s="26" t="n"/>
     </row>
     <row r="53" ht="13" customHeight="1">
       <c r="A53" s="29" t="n">
@@ -4480,10 +4604,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D53" s="31" t="n">
+      <c r="D53" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E53" s="31" t="n">
+      <c r="E53" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F53" s="29" t="n">
@@ -4537,6 +4661,8 @@
       <c r="AZ53" s="32" t="n"/>
       <c r="BA53" s="32" t="n"/>
       <c r="BB53" s="26" t="n"/>
+      <c r="BC53" s="26" t="n"/>
+      <c r="BD53" s="26" t="n"/>
     </row>
     <row r="54" ht="13" customHeight="1">
       <c r="A54" s="29" t="n">
@@ -4552,10 +4678,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D54" s="31" t="n">
+      <c r="D54" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E54" s="31" t="n">
+      <c r="E54" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F54" s="29" t="n">
@@ -4609,6 +4735,8 @@
       <c r="AZ54" s="32" t="n"/>
       <c r="BA54" s="32" t="n"/>
       <c r="BB54" s="26" t="n"/>
+      <c r="BC54" s="26" t="n"/>
+      <c r="BD54" s="26" t="n"/>
     </row>
     <row r="55" ht="13" customHeight="1">
       <c r="A55" s="29" t="n">
@@ -4624,10 +4752,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D55" s="31" t="n">
+      <c r="D55" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E55" s="31" t="n">
+      <c r="E55" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F55" s="29" t="n">
@@ -4681,6 +4809,8 @@
       <c r="AZ55" s="32" t="n"/>
       <c r="BA55" s="32" t="n"/>
       <c r="BB55" s="26" t="n"/>
+      <c r="BC55" s="26" t="n"/>
+      <c r="BD55" s="26" t="n"/>
     </row>
     <row r="56" ht="13" customHeight="1">
       <c r="A56" s="29" t="n">
@@ -4696,10 +4826,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D56" s="31" t="n">
+      <c r="D56" s="73" t="n">
         <v>46104</v>
       </c>
-      <c r="E56" s="31" t="n">
+      <c r="E56" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F56" s="29" t="n">
@@ -4757,6 +4887,8 @@
       <c r="AZ56" s="32" t="n"/>
       <c r="BA56" s="32" t="n"/>
       <c r="BB56" s="26" t="n"/>
+      <c r="BC56" s="26" t="n"/>
+      <c r="BD56" s="26" t="n"/>
     </row>
     <row r="57" ht="13" customHeight="1">
       <c r="A57" s="29" t="n">
@@ -4772,10 +4904,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D57" s="31" t="n">
+      <c r="D57" s="73" t="n">
         <v>46102</v>
       </c>
-      <c r="E57" s="31" t="n">
+      <c r="E57" s="73" t="n">
         <v>46103</v>
       </c>
       <c r="F57" s="29" t="n">
@@ -4829,6 +4961,8 @@
       <c r="AZ57" s="32" t="n"/>
       <c r="BA57" s="32" t="n"/>
       <c r="BB57" s="26" t="n"/>
+      <c r="BC57" s="26" t="n"/>
+      <c r="BD57" s="26" t="n"/>
     </row>
     <row r="58" ht="13" customHeight="1">
       <c r="A58" s="29" t="n">
@@ -4844,10 +4978,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D58" s="31" t="n">
+      <c r="D58" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E58" s="31" t="n">
+      <c r="E58" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F58" s="29" t="n">
@@ -4901,6 +5035,8 @@
       <c r="AZ58" s="32" t="n"/>
       <c r="BA58" s="32" t="n"/>
       <c r="BB58" s="26" t="n"/>
+      <c r="BC58" s="26" t="n"/>
+      <c r="BD58" s="26" t="n"/>
     </row>
     <row r="59" ht="13" customHeight="1">
       <c r="A59" s="29" t="n">
@@ -4916,10 +5052,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D59" s="31" t="n">
+      <c r="D59" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E59" s="31" t="n">
+      <c r="E59" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F59" s="29" t="n">
@@ -4973,6 +5109,8 @@
       <c r="AZ59" s="32" t="n"/>
       <c r="BA59" s="32" t="n"/>
       <c r="BB59" s="26" t="n"/>
+      <c r="BC59" s="26" t="n"/>
+      <c r="BD59" s="26" t="n"/>
     </row>
     <row r="60" ht="13" customHeight="1">
       <c r="A60" s="29" t="n">
@@ -4988,10 +5126,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D60" s="31" t="n">
+      <c r="D60" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E60" s="31" t="n">
+      <c r="E60" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F60" s="29" t="n">
@@ -5045,6 +5183,8 @@
       <c r="AZ60" s="32" t="n"/>
       <c r="BA60" s="32" t="n"/>
       <c r="BB60" s="26" t="n"/>
+      <c r="BC60" s="26" t="n"/>
+      <c r="BD60" s="26" t="n"/>
     </row>
     <row r="61" ht="13" customHeight="1">
       <c r="A61" s="29" t="n">
@@ -5060,10 +5200,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D61" s="31" t="n">
+      <c r="D61" s="73" t="n">
         <v>46104</v>
       </c>
-      <c r="E61" s="31" t="n">
+      <c r="E61" s="73" t="n">
         <v>46105</v>
       </c>
       <c r="F61" s="29" t="n">
@@ -5117,6 +5257,8 @@
       <c r="AZ61" s="32" t="n"/>
       <c r="BA61" s="32" t="n"/>
       <c r="BB61" s="26" t="n"/>
+      <c r="BC61" s="26" t="n"/>
+      <c r="BD61" s="26" t="n"/>
     </row>
     <row r="62" ht="13" customHeight="1">
       <c r="A62" s="29" t="n">
@@ -5132,10 +5274,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D62" s="31" t="n">
+      <c r="D62" s="73" t="n">
         <v>46103</v>
       </c>
-      <c r="E62" s="31" t="n">
+      <c r="E62" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F62" s="29" t="n">
@@ -5189,6 +5331,8 @@
       <c r="AZ62" s="32" t="n"/>
       <c r="BA62" s="32" t="n"/>
       <c r="BB62" s="26" t="n"/>
+      <c r="BC62" s="26" t="n"/>
+      <c r="BD62" s="26" t="n"/>
     </row>
     <row r="63" ht="13" customHeight="1">
       <c r="A63" s="29" t="n">
@@ -5204,10 +5348,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D63" s="31" t="n">
+      <c r="D63" s="73" t="n">
         <v>46104</v>
       </c>
-      <c r="E63" s="31" t="n">
+      <c r="E63" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F63" s="29" t="n">
@@ -5265,6 +5409,8 @@
       <c r="AZ63" s="32" t="n"/>
       <c r="BA63" s="32" t="n"/>
       <c r="BB63" s="26" t="n"/>
+      <c r="BC63" s="26" t="n"/>
+      <c r="BD63" s="26" t="n"/>
     </row>
     <row r="64" ht="13" customHeight="1">
       <c r="A64" s="29" t="n">
@@ -5280,10 +5426,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D64" s="31" t="n">
+      <c r="D64" s="73" t="n">
         <v>46104</v>
       </c>
-      <c r="E64" s="31" t="n">
+      <c r="E64" s="73" t="n">
         <v>46104</v>
       </c>
       <c r="F64" s="29" t="n">
@@ -5341,6 +5487,8 @@
       <c r="AZ64" s="32" t="n"/>
       <c r="BA64" s="32" t="n"/>
       <c r="BB64" s="26" t="n"/>
+      <c r="BC64" s="26" t="n"/>
+      <c r="BD64" s="26" t="n"/>
     </row>
     <row r="65" ht="13" customHeight="1">
       <c r="A65" s="29" t="n">
@@ -5356,10 +5504,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D65" s="31" t="n">
+      <c r="D65" s="73" t="n">
         <v>46104</v>
       </c>
-      <c r="E65" s="31" t="n">
+      <c r="E65" s="73" t="n">
         <v>46106</v>
       </c>
       <c r="F65" s="29" t="n">
@@ -5413,6 +5561,8 @@
       <c r="AZ65" s="32" t="n"/>
       <c r="BA65" s="32" t="n"/>
       <c r="BB65" s="26" t="n"/>
+      <c r="BC65" s="26" t="n"/>
+      <c r="BD65" s="26" t="n"/>
     </row>
     <row r="66" ht="13" customHeight="1">
       <c r="A66" s="29" t="n">
@@ -5428,10 +5578,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D66" s="31" t="n">
+      <c r="D66" s="73" t="n">
         <v>46105</v>
       </c>
-      <c r="E66" s="31" t="n">
+      <c r="E66" s="73" t="n">
         <v>46106</v>
       </c>
       <c r="F66" s="29" t="n">
@@ -5485,6 +5635,8 @@
       <c r="AZ66" s="32" t="n"/>
       <c r="BA66" s="32" t="n"/>
       <c r="BB66" s="26" t="n"/>
+      <c r="BC66" s="26" t="n"/>
+      <c r="BD66" s="26" t="n"/>
     </row>
     <row r="67" ht="13" customHeight="1">
       <c r="A67" s="29" t="n">
@@ -5500,10 +5652,10 @@
           <t>Ph.1</t>
         </is>
       </c>
-      <c r="D67" s="31" t="n">
+      <c r="D67" s="73" t="n">
         <v>46105</v>
       </c>
-      <c r="E67" s="31" t="n">
+      <c r="E67" s="73" t="n">
         <v>46106</v>
       </c>
       <c r="F67" s="29" t="n">
@@ -5557,6 +5709,8 @@
       <c r="AZ67" s="32" t="n"/>
       <c r="BA67" s="32" t="n"/>
       <c r="BB67" s="26" t="n"/>
+      <c r="BC67" s="26" t="n"/>
+      <c r="BD67" s="26" t="n"/>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
@@ -5612,6 +5766,8 @@
       <c r="AZ68" s="35" t="n"/>
       <c r="BA68" s="35" t="n"/>
       <c r="BB68" s="35" t="n"/>
+      <c r="BC68" s="35" t="n"/>
+      <c r="BD68" s="35" t="n"/>
     </row>
     <row r="69" ht="13" customHeight="1">
       <c r="A69" s="36" t="n">
@@ -5627,10 +5783,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D69" s="38" t="n">
+      <c r="D69" s="74" t="n">
         <v>46103</v>
       </c>
-      <c r="E69" s="38" t="n">
+      <c r="E69" s="74" t="n">
         <v>46104</v>
       </c>
       <c r="F69" s="36" t="n">
@@ -5684,6 +5840,8 @@
       <c r="AZ69" s="39" t="n"/>
       <c r="BA69" s="39" t="n"/>
       <c r="BB69" s="26" t="n"/>
+      <c r="BC69" s="26" t="n"/>
+      <c r="BD69" s="26" t="n"/>
     </row>
     <row r="70" ht="13" customHeight="1">
       <c r="A70" s="36" t="n">
@@ -5699,10 +5857,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D70" s="38" t="n">
+      <c r="D70" s="74" t="n">
         <v>46103</v>
       </c>
-      <c r="E70" s="38" t="n">
+      <c r="E70" s="74" t="n">
         <v>46104</v>
       </c>
       <c r="F70" s="36" t="n">
@@ -5756,6 +5914,8 @@
       <c r="AZ70" s="39" t="n"/>
       <c r="BA70" s="39" t="n"/>
       <c r="BB70" s="26" t="n"/>
+      <c r="BC70" s="26" t="n"/>
+      <c r="BD70" s="26" t="n"/>
     </row>
     <row r="71" ht="13" customHeight="1">
       <c r="A71" s="36" t="n">
@@ -5771,10 +5931,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D71" s="38" t="n">
+      <c r="D71" s="74" t="n">
         <v>46105</v>
       </c>
-      <c r="E71" s="38" t="n">
+      <c r="E71" s="74" t="n">
         <v>46105</v>
       </c>
       <c r="F71" s="36" t="n">
@@ -5832,6 +5992,8 @@
       <c r="AZ71" s="39" t="n"/>
       <c r="BA71" s="39" t="n"/>
       <c r="BB71" s="26" t="n"/>
+      <c r="BC71" s="26" t="n"/>
+      <c r="BD71" s="26" t="n"/>
     </row>
     <row r="72" ht="13" customHeight="1">
       <c r="A72" s="36" t="n">
@@ -5847,10 +6009,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D72" s="38" t="n">
+      <c r="D72" s="74" t="n">
         <v>46105</v>
       </c>
-      <c r="E72" s="38" t="n">
+      <c r="E72" s="74" t="n">
         <v>46105</v>
       </c>
       <c r="F72" s="36" t="n">
@@ -5908,6 +6070,8 @@
       <c r="AZ72" s="39" t="n"/>
       <c r="BA72" s="39" t="n"/>
       <c r="BB72" s="26" t="n"/>
+      <c r="BC72" s="26" t="n"/>
+      <c r="BD72" s="26" t="n"/>
     </row>
     <row r="73" ht="13" customHeight="1">
       <c r="A73" s="36" t="n">
@@ -5923,10 +6087,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D73" s="38" t="n">
+      <c r="D73" s="74" t="n">
         <v>46105</v>
       </c>
-      <c r="E73" s="38" t="n">
+      <c r="E73" s="74" t="n">
         <v>46105</v>
       </c>
       <c r="F73" s="36" t="n">
@@ -5984,6 +6148,8 @@
       <c r="AZ73" s="39" t="n"/>
       <c r="BA73" s="39" t="n"/>
       <c r="BB73" s="26" t="n"/>
+      <c r="BC73" s="26" t="n"/>
+      <c r="BD73" s="26" t="n"/>
     </row>
     <row r="74" ht="13" customHeight="1">
       <c r="A74" s="36" t="n">
@@ -5999,10 +6165,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D74" s="38" t="n">
+      <c r="D74" s="74" t="n">
         <v>46105</v>
       </c>
-      <c r="E74" s="38" t="n">
+      <c r="E74" s="74" t="n">
         <v>46105</v>
       </c>
       <c r="F74" s="36" t="n">
@@ -6060,6 +6226,8 @@
       <c r="AZ74" s="39" t="n"/>
       <c r="BA74" s="39" t="n"/>
       <c r="BB74" s="26" t="n"/>
+      <c r="BC74" s="26" t="n"/>
+      <c r="BD74" s="26" t="n"/>
     </row>
     <row r="75" ht="13" customHeight="1">
       <c r="A75" s="36" t="n">
@@ -6075,10 +6243,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D75" s="38" t="n">
+      <c r="D75" s="74" t="n">
         <v>46105</v>
       </c>
-      <c r="E75" s="38" t="n">
+      <c r="E75" s="74" t="n">
         <v>46105</v>
       </c>
       <c r="F75" s="36" t="n">
@@ -6136,6 +6304,8 @@
       <c r="AZ75" s="39" t="n"/>
       <c r="BA75" s="39" t="n"/>
       <c r="BB75" s="26" t="n"/>
+      <c r="BC75" s="26" t="n"/>
+      <c r="BD75" s="26" t="n"/>
     </row>
     <row r="76" ht="13" customHeight="1">
       <c r="A76" s="36" t="n">
@@ -6151,10 +6321,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D76" s="38" t="n">
+      <c r="D76" s="74" t="n">
         <v>46106</v>
       </c>
-      <c r="E76" s="38" t="n">
+      <c r="E76" s="74" t="n">
         <v>46106</v>
       </c>
       <c r="F76" s="36" t="n">
@@ -6212,6 +6382,8 @@
       <c r="AZ76" s="39" t="n"/>
       <c r="BA76" s="39" t="n"/>
       <c r="BB76" s="26" t="n"/>
+      <c r="BC76" s="26" t="n"/>
+      <c r="BD76" s="26" t="n"/>
     </row>
     <row r="77" ht="13" customHeight="1">
       <c r="A77" s="36" t="n">
@@ -6227,10 +6399,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D77" s="38" t="n">
+      <c r="D77" s="74" t="n">
         <v>46106</v>
       </c>
-      <c r="E77" s="38" t="n">
+      <c r="E77" s="74" t="n">
         <v>46106</v>
       </c>
       <c r="F77" s="36" t="n">
@@ -6288,6 +6460,8 @@
       <c r="AZ77" s="39" t="n"/>
       <c r="BA77" s="39" t="n"/>
       <c r="BB77" s="26" t="n"/>
+      <c r="BC77" s="26" t="n"/>
+      <c r="BD77" s="26" t="n"/>
     </row>
     <row r="78" ht="13" customHeight="1">
       <c r="A78" s="36" t="n">
@@ -6303,10 +6477,10 @@
           <t>Ph.2</t>
         </is>
       </c>
-      <c r="D78" s="38" t="n">
+      <c r="D78" s="74" t="n">
         <v>46107</v>
       </c>
-      <c r="E78" s="38" t="n">
+      <c r="E78" s="74" t="n">
         <v>46107</v>
       </c>
       <c r="F78" s="36" t="n">
@@ -6364,6 +6538,8 @@
       <c r="AZ78" s="39" t="n"/>
       <c r="BA78" s="39" t="n"/>
       <c r="BB78" s="26" t="n"/>
+      <c r="BC78" s="26" t="n"/>
+      <c r="BD78" s="26" t="n"/>
     </row>
     <row r="79" ht="14" customHeight="1">
       <c r="A79" s="7" t="inlineStr">
@@ -6419,6 +6595,8 @@
       <c r="AZ79" s="42" t="n"/>
       <c r="BA79" s="42" t="n"/>
       <c r="BB79" s="42" t="n"/>
+      <c r="BC79" s="42" t="n"/>
+      <c r="BD79" s="42" t="n"/>
     </row>
     <row r="80" ht="13" customHeight="1">
       <c r="A80" s="43" t="n">
@@ -6434,10 +6612,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D80" s="45" t="n">
+      <c r="D80" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E80" s="45" t="n">
+      <c r="E80" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F80" s="43" t="n">
@@ -6491,6 +6669,8 @@
       <c r="AZ80" s="46" t="n"/>
       <c r="BA80" s="46" t="n"/>
       <c r="BB80" s="26" t="n"/>
+      <c r="BC80" s="26" t="n"/>
+      <c r="BD80" s="26" t="n"/>
     </row>
     <row r="81" ht="13" customHeight="1">
       <c r="A81" s="43" t="n">
@@ -6506,10 +6686,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D81" s="45" t="n">
+      <c r="D81" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E81" s="45" t="n">
+      <c r="E81" s="75" t="n">
         <v>46109</v>
       </c>
       <c r="F81" s="43" t="n">
@@ -6563,6 +6743,8 @@
       <c r="AZ81" s="46" t="n"/>
       <c r="BA81" s="46" t="n"/>
       <c r="BB81" s="26" t="n"/>
+      <c r="BC81" s="26" t="n"/>
+      <c r="BD81" s="26" t="n"/>
     </row>
     <row r="82" ht="13" customHeight="1">
       <c r="A82" s="43" t="n">
@@ -6578,10 +6760,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D82" s="45" t="n">
+      <c r="D82" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E82" s="45" t="n">
+      <c r="E82" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F82" s="43" t="n">
@@ -6635,6 +6817,8 @@
       <c r="AZ82" s="46" t="n"/>
       <c r="BA82" s="46" t="n"/>
       <c r="BB82" s="26" t="n"/>
+      <c r="BC82" s="26" t="n"/>
+      <c r="BD82" s="26" t="n"/>
     </row>
     <row r="83" ht="13" customHeight="1">
       <c r="A83" s="43" t="n">
@@ -6650,10 +6834,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D83" s="45" t="n">
+      <c r="D83" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E83" s="45" t="n">
+      <c r="E83" s="75" t="n">
         <v>46109</v>
       </c>
       <c r="F83" s="43" t="n">
@@ -6707,6 +6891,8 @@
       <c r="AZ83" s="46" t="n"/>
       <c r="BA83" s="46" t="n"/>
       <c r="BB83" s="26" t="n"/>
+      <c r="BC83" s="26" t="n"/>
+      <c r="BD83" s="26" t="n"/>
     </row>
     <row r="84" ht="13" customHeight="1">
       <c r="A84" s="43" t="n">
@@ -6722,10 +6908,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D84" s="45" t="n">
+      <c r="D84" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E84" s="45" t="n">
+      <c r="E84" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F84" s="43" t="n">
@@ -6779,6 +6965,8 @@
       <c r="AZ84" s="46" t="n"/>
       <c r="BA84" s="46" t="n"/>
       <c r="BB84" s="26" t="n"/>
+      <c r="BC84" s="26" t="n"/>
+      <c r="BD84" s="26" t="n"/>
     </row>
     <row r="85" ht="13" customHeight="1">
       <c r="A85" s="43" t="n">
@@ -6794,10 +6982,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D85" s="45" t="n">
+      <c r="D85" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E85" s="45" t="n">
+      <c r="E85" s="75" t="n">
         <v>46108</v>
       </c>
       <c r="F85" s="43" t="n">
@@ -6855,6 +7043,8 @@
       <c r="AZ85" s="46" t="n"/>
       <c r="BA85" s="46" t="n"/>
       <c r="BB85" s="26" t="n"/>
+      <c r="BC85" s="26" t="n"/>
+      <c r="BD85" s="26" t="n"/>
     </row>
     <row r="86" ht="13" customHeight="1">
       <c r="A86" s="43" t="n">
@@ -6870,10 +7060,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D86" s="45" t="n">
+      <c r="D86" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E86" s="45" t="n">
+      <c r="E86" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F86" s="43" t="n">
@@ -6927,6 +7117,8 @@
       <c r="AZ86" s="46" t="n"/>
       <c r="BA86" s="46" t="n"/>
       <c r="BB86" s="26" t="n"/>
+      <c r="BC86" s="26" t="n"/>
+      <c r="BD86" s="26" t="n"/>
     </row>
     <row r="87" ht="13" customHeight="1">
       <c r="A87" s="43" t="n">
@@ -6942,10 +7134,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D87" s="45" t="n">
+      <c r="D87" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E87" s="45" t="n">
+      <c r="E87" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F87" s="43" t="n">
@@ -6999,6 +7191,8 @@
       <c r="AZ87" s="46" t="n"/>
       <c r="BA87" s="46" t="n"/>
       <c r="BB87" s="26" t="n"/>
+      <c r="BC87" s="26" t="n"/>
+      <c r="BD87" s="26" t="n"/>
     </row>
     <row r="88" ht="13" customHeight="1">
       <c r="A88" s="43" t="n">
@@ -7014,10 +7208,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D88" s="45" t="n">
+      <c r="D88" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E88" s="45" t="n">
+      <c r="E88" s="75" t="n">
         <v>46109</v>
       </c>
       <c r="F88" s="43" t="n">
@@ -7075,6 +7269,8 @@
       <c r="AZ88" s="46" t="n"/>
       <c r="BA88" s="46" t="n"/>
       <c r="BB88" s="26" t="n"/>
+      <c r="BC88" s="26" t="n"/>
+      <c r="BD88" s="26" t="n"/>
     </row>
     <row r="89" ht="13" customHeight="1">
       <c r="A89" s="43" t="n">
@@ -7090,10 +7286,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D89" s="45" t="n">
+      <c r="D89" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E89" s="45" t="n">
+      <c r="E89" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F89" s="43" t="n">
@@ -7147,6 +7343,8 @@
       <c r="AZ89" s="46" t="n"/>
       <c r="BA89" s="46" t="n"/>
       <c r="BB89" s="26" t="n"/>
+      <c r="BC89" s="26" t="n"/>
+      <c r="BD89" s="26" t="n"/>
     </row>
     <row r="90" ht="13" customHeight="1">
       <c r="A90" s="43" t="n">
@@ -7162,10 +7360,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D90" s="45" t="n">
+      <c r="D90" s="75" t="n">
         <v>46110</v>
       </c>
-      <c r="E90" s="45" t="n">
+      <c r="E90" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F90" s="43" t="n">
@@ -7219,6 +7417,8 @@
       <c r="AZ90" s="46" t="n"/>
       <c r="BA90" s="46" t="n"/>
       <c r="BB90" s="26" t="n"/>
+      <c r="BC90" s="26" t="n"/>
+      <c r="BD90" s="26" t="n"/>
     </row>
     <row r="91" ht="13" customHeight="1">
       <c r="A91" s="43" t="n">
@@ -7234,10 +7434,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D91" s="45" t="n">
+      <c r="D91" s="75" t="n">
         <v>46110</v>
       </c>
-      <c r="E91" s="45" t="n">
+      <c r="E91" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F91" s="43" t="n">
@@ -7291,6 +7491,8 @@
       <c r="AZ91" s="46" t="n"/>
       <c r="BA91" s="46" t="n"/>
       <c r="BB91" s="26" t="n"/>
+      <c r="BC91" s="26" t="n"/>
+      <c r="BD91" s="26" t="n"/>
     </row>
     <row r="92" ht="13" customHeight="1">
       <c r="A92" s="43" t="n">
@@ -7306,10 +7508,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D92" s="45" t="n">
+      <c r="D92" s="75" t="n">
         <v>46110</v>
       </c>
-      <c r="E92" s="45" t="n">
+      <c r="E92" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F92" s="43" t="n">
@@ -7363,6 +7565,8 @@
       <c r="AZ92" s="46" t="n"/>
       <c r="BA92" s="46" t="n"/>
       <c r="BB92" s="26" t="n"/>
+      <c r="BC92" s="26" t="n"/>
+      <c r="BD92" s="26" t="n"/>
     </row>
     <row r="93" ht="13" customHeight="1">
       <c r="A93" s="43" t="n">
@@ -7378,10 +7582,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D93" s="45" t="n">
+      <c r="D93" s="75" t="n">
         <v>46111</v>
       </c>
-      <c r="E93" s="45" t="n">
+      <c r="E93" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F93" s="43" t="n">
@@ -7439,6 +7643,8 @@
       <c r="AZ93" s="46" t="n"/>
       <c r="BA93" s="46" t="n"/>
       <c r="BB93" s="26" t="n"/>
+      <c r="BC93" s="26" t="n"/>
+      <c r="BD93" s="26" t="n"/>
     </row>
     <row r="94" ht="13" customHeight="1">
       <c r="A94" s="43" t="n">
@@ -7454,10 +7660,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D94" s="45" t="n">
+      <c r="D94" s="75" t="n">
         <v>46110</v>
       </c>
-      <c r="E94" s="45" t="n">
+      <c r="E94" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F94" s="43" t="n">
@@ -7511,6 +7717,8 @@
       <c r="AZ94" s="46" t="n"/>
       <c r="BA94" s="46" t="n"/>
       <c r="BB94" s="26" t="n"/>
+      <c r="BC94" s="26" t="n"/>
+      <c r="BD94" s="26" t="n"/>
     </row>
     <row r="95" ht="13" customHeight="1">
       <c r="A95" s="43" t="n">
@@ -7526,10 +7734,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D95" s="45" t="n">
+      <c r="D95" s="75" t="n">
         <v>46111</v>
       </c>
-      <c r="E95" s="45" t="n">
+      <c r="E95" s="75" t="n">
         <v>46112</v>
       </c>
       <c r="F95" s="43" t="n">
@@ -7583,6 +7791,8 @@
       <c r="AZ95" s="46" t="n"/>
       <c r="BA95" s="46" t="n"/>
       <c r="BB95" s="26" t="n"/>
+      <c r="BC95" s="26" t="n"/>
+      <c r="BD95" s="26" t="n"/>
     </row>
     <row r="96" ht="13" customHeight="1">
       <c r="A96" s="43" t="n">
@@ -7598,10 +7808,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D96" s="45" t="n">
+      <c r="D96" s="75" t="n">
         <v>46111</v>
       </c>
-      <c r="E96" s="45" t="n">
+      <c r="E96" s="75" t="n">
         <v>46112</v>
       </c>
       <c r="F96" s="43" t="n">
@@ -7655,6 +7865,8 @@
       <c r="AZ96" s="46" t="n"/>
       <c r="BA96" s="46" t="n"/>
       <c r="BB96" s="26" t="n"/>
+      <c r="BC96" s="26" t="n"/>
+      <c r="BD96" s="26" t="n"/>
     </row>
     <row r="97" ht="13" customHeight="1">
       <c r="A97" s="43" t="n">
@@ -7670,10 +7882,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D97" s="45" t="n">
+      <c r="D97" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E97" s="45" t="n">
+      <c r="E97" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F97" s="43" t="n">
@@ -7727,6 +7939,8 @@
       <c r="AZ97" s="46" t="n"/>
       <c r="BA97" s="46" t="n"/>
       <c r="BB97" s="26" t="n"/>
+      <c r="BC97" s="26" t="n"/>
+      <c r="BD97" s="26" t="n"/>
     </row>
     <row r="98" ht="13" customHeight="1">
       <c r="A98" s="43" t="n">
@@ -7742,10 +7956,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D98" s="45" t="n">
+      <c r="D98" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E98" s="45" t="n">
+      <c r="E98" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F98" s="43" t="n">
@@ -7799,6 +8013,8 @@
       <c r="AZ98" s="46" t="n"/>
       <c r="BA98" s="46" t="n"/>
       <c r="BB98" s="26" t="n"/>
+      <c r="BC98" s="26" t="n"/>
+      <c r="BD98" s="26" t="n"/>
     </row>
     <row r="99" ht="13" customHeight="1">
       <c r="A99" s="43" t="n">
@@ -7814,10 +8030,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D99" s="45" t="n">
+      <c r="D99" s="75" t="n">
         <v>46110</v>
       </c>
-      <c r="E99" s="45" t="n">
+      <c r="E99" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F99" s="43" t="n">
@@ -7871,6 +8087,8 @@
       <c r="AZ99" s="46" t="n"/>
       <c r="BA99" s="46" t="n"/>
       <c r="BB99" s="26" t="n"/>
+      <c r="BC99" s="26" t="n"/>
+      <c r="BD99" s="26" t="n"/>
     </row>
     <row r="100" ht="13" customHeight="1">
       <c r="A100" s="43" t="n">
@@ -7886,10 +8104,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D100" s="45" t="n">
+      <c r="D100" s="75" t="n">
         <v>46108</v>
       </c>
-      <c r="E100" s="45" t="n">
+      <c r="E100" s="75" t="n">
         <v>46109</v>
       </c>
       <c r="F100" s="43" t="n">
@@ -7943,6 +8161,8 @@
       <c r="AZ100" s="46" t="n"/>
       <c r="BA100" s="46" t="n"/>
       <c r="BB100" s="26" t="n"/>
+      <c r="BC100" s="26" t="n"/>
+      <c r="BD100" s="26" t="n"/>
     </row>
     <row r="101" ht="13" customHeight="1">
       <c r="A101" s="43" t="n">
@@ -7958,10 +8178,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D101" s="45" t="n">
+      <c r="D101" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E101" s="45" t="n">
+      <c r="E101" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F101" s="43" t="n">
@@ -8015,6 +8235,8 @@
       <c r="AZ101" s="46" t="n"/>
       <c r="BA101" s="46" t="n"/>
       <c r="BB101" s="26" t="n"/>
+      <c r="BC101" s="26" t="n"/>
+      <c r="BD101" s="26" t="n"/>
     </row>
     <row r="102" ht="13" customHeight="1">
       <c r="A102" s="43" t="n">
@@ -8030,10 +8252,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D102" s="45" t="n">
+      <c r="D102" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E102" s="45" t="n">
+      <c r="E102" s="75" t="n">
         <v>46110</v>
       </c>
       <c r="F102" s="43" t="n">
@@ -8087,6 +8309,8 @@
       <c r="AZ102" s="46" t="n"/>
       <c r="BA102" s="46" t="n"/>
       <c r="BB102" s="26" t="n"/>
+      <c r="BC102" s="26" t="n"/>
+      <c r="BD102" s="26" t="n"/>
     </row>
     <row r="103" ht="13" customHeight="1">
       <c r="A103" s="43" t="n">
@@ -8102,10 +8326,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D103" s="45" t="n">
+      <c r="D103" s="75" t="n">
         <v>46109</v>
       </c>
-      <c r="E103" s="45" t="n">
+      <c r="E103" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F103" s="43" t="n">
@@ -8159,6 +8383,8 @@
       <c r="AZ103" s="46" t="n"/>
       <c r="BA103" s="46" t="n"/>
       <c r="BB103" s="26" t="n"/>
+      <c r="BC103" s="26" t="n"/>
+      <c r="BD103" s="26" t="n"/>
     </row>
     <row r="104" ht="13" customHeight="1">
       <c r="A104" s="43" t="n">
@@ -8174,10 +8400,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D104" s="45" t="n">
+      <c r="D104" s="75" t="n">
         <v>46110</v>
       </c>
-      <c r="E104" s="45" t="n">
+      <c r="E104" s="75" t="n">
         <v>46111</v>
       </c>
       <c r="F104" s="43" t="n">
@@ -8231,6 +8457,8 @@
       <c r="AZ104" s="46" t="n"/>
       <c r="BA104" s="46" t="n"/>
       <c r="BB104" s="26" t="n"/>
+      <c r="BC104" s="26" t="n"/>
+      <c r="BD104" s="26" t="n"/>
     </row>
     <row r="105" ht="13" customHeight="1">
       <c r="A105" s="43" t="n">
@@ -8246,10 +8474,10 @@
           <t>Ph.3</t>
         </is>
       </c>
-      <c r="D105" s="45" t="n">
+      <c r="D105" s="75" t="n">
         <v>46111</v>
       </c>
-      <c r="E105" s="45" t="n">
+      <c r="E105" s="75" t="n">
         <v>46112</v>
       </c>
       <c r="F105" s="43" t="n">
@@ -8303,6 +8531,8 @@
       <c r="AZ105" s="46" t="n"/>
       <c r="BA105" s="46" t="n"/>
       <c r="BB105" s="26" t="n"/>
+      <c r="BC105" s="26" t="n"/>
+      <c r="BD105" s="26" t="n"/>
     </row>
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="8" t="inlineStr">
@@ -8358,6 +8588,8 @@
       <c r="AZ106" s="49" t="n"/>
       <c r="BA106" s="49" t="n"/>
       <c r="BB106" s="49" t="n"/>
+      <c r="BC106" s="49" t="n"/>
+      <c r="BD106" s="49" t="n"/>
     </row>
     <row r="107" ht="13" customHeight="1">
       <c r="A107" s="50" t="n">
@@ -8373,10 +8605,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D107" s="52" t="n">
+      <c r="D107" s="76" t="n">
         <v>46125</v>
       </c>
-      <c r="E107" s="52" t="n">
+      <c r="E107" s="76" t="n">
         <v>46127</v>
       </c>
       <c r="F107" s="50" t="n">
@@ -8430,6 +8662,8 @@
       <c r="AZ107" s="53" t="n"/>
       <c r="BA107" s="53" t="n"/>
       <c r="BB107" s="26" t="n"/>
+      <c r="BC107" s="26" t="n"/>
+      <c r="BD107" s="26" t="n"/>
     </row>
     <row r="108" ht="13" customHeight="1">
       <c r="A108" s="50" t="n">
@@ -8445,10 +8679,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D108" s="52" t="n">
+      <c r="D108" s="76" t="n">
         <v>46125</v>
       </c>
-      <c r="E108" s="52" t="n">
+      <c r="E108" s="76" t="n">
         <v>46126</v>
       </c>
       <c r="F108" s="50" t="n">
@@ -8502,6 +8736,8 @@
       <c r="AZ108" s="53" t="n"/>
       <c r="BA108" s="53" t="n"/>
       <c r="BB108" s="26" t="n"/>
+      <c r="BC108" s="26" t="n"/>
+      <c r="BD108" s="26" t="n"/>
     </row>
     <row r="109" ht="13" customHeight="1">
       <c r="A109" s="50" t="n">
@@ -8517,10 +8753,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D109" s="52" t="n">
+      <c r="D109" s="76" t="n">
         <v>46125</v>
       </c>
-      <c r="E109" s="52" t="n">
+      <c r="E109" s="76" t="n">
         <v>46126</v>
       </c>
       <c r="F109" s="50" t="n">
@@ -8574,6 +8810,8 @@
       <c r="AZ109" s="53" t="n"/>
       <c r="BA109" s="53" t="n"/>
       <c r="BB109" s="26" t="n"/>
+      <c r="BC109" s="26" t="n"/>
+      <c r="BD109" s="26" t="n"/>
     </row>
     <row r="110" ht="13" customHeight="1">
       <c r="A110" s="50" t="n">
@@ -8589,10 +8827,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D110" s="52" t="n">
+      <c r="D110" s="76" t="n">
         <v>46126</v>
       </c>
-      <c r="E110" s="52" t="n">
+      <c r="E110" s="76" t="n">
         <v>46127</v>
       </c>
       <c r="F110" s="50" t="n">
@@ -8646,6 +8884,8 @@
       <c r="AZ110" s="53" t="n"/>
       <c r="BA110" s="53" t="n"/>
       <c r="BB110" s="26" t="n"/>
+      <c r="BC110" s="26" t="n"/>
+      <c r="BD110" s="26" t="n"/>
     </row>
     <row r="111" ht="13" customHeight="1">
       <c r="A111" s="50" t="n">
@@ -8661,10 +8901,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D111" s="52" t="n">
+      <c r="D111" s="76" t="n">
         <v>46126</v>
       </c>
-      <c r="E111" s="52" t="n">
+      <c r="E111" s="76" t="n">
         <v>46127</v>
       </c>
       <c r="F111" s="50" t="n">
@@ -8718,6 +8958,8 @@
       <c r="AZ111" s="53" t="n"/>
       <c r="BA111" s="53" t="n"/>
       <c r="BB111" s="26" t="n"/>
+      <c r="BC111" s="26" t="n"/>
+      <c r="BD111" s="26" t="n"/>
     </row>
     <row r="112" ht="13" customHeight="1">
       <c r="A112" s="50" t="n">
@@ -8733,10 +8975,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D112" s="52" t="n">
+      <c r="D112" s="76" t="n">
         <v>46125</v>
       </c>
-      <c r="E112" s="52" t="n">
+      <c r="E112" s="76" t="n">
         <v>46127</v>
       </c>
       <c r="F112" s="50" t="n">
@@ -8790,6 +9032,8 @@
       <c r="AZ112" s="53" t="n"/>
       <c r="BA112" s="53" t="n"/>
       <c r="BB112" s="26" t="n"/>
+      <c r="BC112" s="26" t="n"/>
+      <c r="BD112" s="26" t="n"/>
     </row>
     <row r="113" ht="13" customHeight="1">
       <c r="A113" s="50" t="n">
@@ -8805,10 +9049,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D113" s="52" t="n">
+      <c r="D113" s="76" t="n">
         <v>46127</v>
       </c>
-      <c r="E113" s="52" t="n">
+      <c r="E113" s="76" t="n">
         <v>46127</v>
       </c>
       <c r="F113" s="50" t="n">
@@ -8866,6 +9110,8 @@
       <c r="AZ113" s="53" t="n"/>
       <c r="BA113" s="53" t="n"/>
       <c r="BB113" s="26" t="n"/>
+      <c r="BC113" s="26" t="n"/>
+      <c r="BD113" s="26" t="n"/>
     </row>
     <row r="114" ht="13" customHeight="1">
       <c r="A114" s="50" t="n">
@@ -8881,10 +9127,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D114" s="52" t="n">
+      <c r="D114" s="76" t="n">
         <v>46127</v>
       </c>
-      <c r="E114" s="52" t="n">
+      <c r="E114" s="76" t="n">
         <v>46128</v>
       </c>
       <c r="F114" s="50" t="n">
@@ -8938,6 +9184,8 @@
       <c r="AZ114" s="53" t="n"/>
       <c r="BA114" s="53" t="n"/>
       <c r="BB114" s="26" t="n"/>
+      <c r="BC114" s="26" t="n"/>
+      <c r="BD114" s="26" t="n"/>
     </row>
     <row r="115" ht="13" customHeight="1">
       <c r="A115" s="50" t="n">
@@ -8953,10 +9201,10 @@
           <t>Ph.4</t>
         </is>
       </c>
-      <c r="D115" s="52" t="n">
+      <c r="D115" s="76" t="n">
         <v>46127</v>
       </c>
-      <c r="E115" s="52" t="n">
+      <c r="E115" s="76" t="n">
         <v>46128</v>
       </c>
       <c r="F115" s="50" t="n">
@@ -9010,6 +9258,8 @@
       <c r="AZ115" s="53" t="n"/>
       <c r="BA115" s="53" t="n"/>
       <c r="BB115" s="26" t="n"/>
+      <c r="BC115" s="26" t="n"/>
+      <c r="BD115" s="26" t="n"/>
     </row>
     <row r="116" ht="14" customHeight="1">
       <c r="A116" s="9" t="inlineStr">
@@ -9065,6 +9315,8 @@
       <c r="AZ116" s="56" t="n"/>
       <c r="BA116" s="56" t="n"/>
       <c r="BB116" s="56" t="n"/>
+      <c r="BC116" s="56" t="n"/>
+      <c r="BD116" s="56" t="n"/>
     </row>
     <row r="117" ht="13" customHeight="1">
       <c r="A117" s="21" t="n">
@@ -9080,10 +9332,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D117" s="23" t="n">
+      <c r="D117" s="72" t="n">
         <v>46129</v>
       </c>
-      <c r="E117" s="23" t="n">
+      <c r="E117" s="72" t="n">
         <v>46130</v>
       </c>
       <c r="F117" s="21" t="n">
@@ -9137,6 +9389,8 @@
       <c r="AZ117" s="24" t="n"/>
       <c r="BA117" s="24" t="n"/>
       <c r="BB117" s="26" t="n"/>
+      <c r="BC117" s="26" t="n"/>
+      <c r="BD117" s="26" t="n"/>
     </row>
     <row r="118" ht="13" customHeight="1">
       <c r="A118" s="21" t="n">
@@ -9152,10 +9406,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D118" s="23" t="n">
+      <c r="D118" s="72" t="n">
         <v>46129</v>
       </c>
-      <c r="E118" s="23" t="n">
+      <c r="E118" s="72" t="n">
         <v>46130</v>
       </c>
       <c r="F118" s="21" t="n">
@@ -9209,6 +9463,8 @@
       <c r="AZ118" s="24" t="n"/>
       <c r="BA118" s="24" t="n"/>
       <c r="BB118" s="26" t="n"/>
+      <c r="BC118" s="26" t="n"/>
+      <c r="BD118" s="26" t="n"/>
     </row>
     <row r="119" ht="13" customHeight="1">
       <c r="A119" s="21" t="n">
@@ -9224,10 +9480,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D119" s="23" t="n">
+      <c r="D119" s="72" t="n">
         <v>46130</v>
       </c>
-      <c r="E119" s="23" t="n">
+      <c r="E119" s="72" t="n">
         <v>46130</v>
       </c>
       <c r="F119" s="21" t="n">
@@ -9285,6 +9541,8 @@
       <c r="AZ119" s="24" t="n"/>
       <c r="BA119" s="24" t="n"/>
       <c r="BB119" s="26" t="n"/>
+      <c r="BC119" s="26" t="n"/>
+      <c r="BD119" s="26" t="n"/>
     </row>
     <row r="120" ht="13" customHeight="1">
       <c r="A120" s="21" t="n">
@@ -9300,10 +9558,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D120" s="23" t="n">
+      <c r="D120" s="72" t="n">
         <v>46129</v>
       </c>
-      <c r="E120" s="23" t="n">
+      <c r="E120" s="72" t="n">
         <v>46130</v>
       </c>
       <c r="F120" s="21" t="n">
@@ -9357,6 +9615,8 @@
       <c r="AZ120" s="24" t="n"/>
       <c r="BA120" s="24" t="n"/>
       <c r="BB120" s="26" t="n"/>
+      <c r="BC120" s="26" t="n"/>
+      <c r="BD120" s="26" t="n"/>
     </row>
     <row r="121" ht="13" customHeight="1">
       <c r="A121" s="21" t="n">
@@ -9372,10 +9632,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D121" s="23" t="n">
+      <c r="D121" s="72" t="n">
         <v>46130</v>
       </c>
-      <c r="E121" s="23" t="n">
+      <c r="E121" s="72" t="n">
         <v>46131</v>
       </c>
       <c r="F121" s="21" t="n">
@@ -9429,6 +9689,8 @@
       <c r="AZ121" s="24" t="n"/>
       <c r="BA121" s="24" t="n"/>
       <c r="BB121" s="26" t="n"/>
+      <c r="BC121" s="26" t="n"/>
+      <c r="BD121" s="26" t="n"/>
     </row>
     <row r="122" ht="13" customHeight="1">
       <c r="A122" s="21" t="n">
@@ -9444,10 +9706,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D122" s="23" t="n">
+      <c r="D122" s="72" t="n">
         <v>46130</v>
       </c>
-      <c r="E122" s="23" t="n">
+      <c r="E122" s="72" t="n">
         <v>46131</v>
       </c>
       <c r="F122" s="21" t="n">
@@ -9501,6 +9763,8 @@
       <c r="AZ122" s="24" t="n"/>
       <c r="BA122" s="24" t="n"/>
       <c r="BB122" s="26" t="n"/>
+      <c r="BC122" s="26" t="n"/>
+      <c r="BD122" s="26" t="n"/>
     </row>
     <row r="123" ht="13" customHeight="1">
       <c r="A123" s="21" t="n">
@@ -9516,10 +9780,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D123" s="23" t="n">
+      <c r="D123" s="72" t="n">
         <v>46129</v>
       </c>
-      <c r="E123" s="23" t="n">
+      <c r="E123" s="72" t="n">
         <v>46130</v>
       </c>
       <c r="F123" s="21" t="n">
@@ -9573,6 +9837,8 @@
       <c r="AZ123" s="24" t="n"/>
       <c r="BA123" s="24" t="n"/>
       <c r="BB123" s="26" t="n"/>
+      <c r="BC123" s="26" t="n"/>
+      <c r="BD123" s="26" t="n"/>
     </row>
     <row r="124" ht="13" customHeight="1">
       <c r="A124" s="21" t="n">
@@ -9588,10 +9854,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D124" s="23" t="n">
+      <c r="D124" s="72" t="n">
         <v>46131</v>
       </c>
-      <c r="E124" s="23" t="n">
+      <c r="E124" s="72" t="n">
         <v>46131</v>
       </c>
       <c r="F124" s="21" t="n">
@@ -9649,6 +9915,8 @@
       <c r="AZ124" s="24" t="n"/>
       <c r="BA124" s="24" t="n"/>
       <c r="BB124" s="26" t="n"/>
+      <c r="BC124" s="26" t="n"/>
+      <c r="BD124" s="26" t="n"/>
     </row>
     <row r="125" ht="13" customHeight="1">
       <c r="A125" s="21" t="n">
@@ -9664,10 +9932,10 @@
           <t>Ph.5</t>
         </is>
       </c>
-      <c r="D125" s="23" t="n">
+      <c r="D125" s="72" t="n">
         <v>46130</v>
       </c>
-      <c r="E125" s="23" t="n">
+      <c r="E125" s="72" t="n">
         <v>46131</v>
       </c>
       <c r="F125" s="21" t="n">
@@ -9721,6 +9989,8 @@
       <c r="AZ125" s="24" t="n"/>
       <c r="BA125" s="24" t="n"/>
       <c r="BB125" s="26" t="n"/>
+      <c r="BC125" s="26" t="n"/>
+      <c r="BD125" s="26" t="n"/>
     </row>
     <row r="126" ht="14" customHeight="1">
       <c r="A126" s="10" t="inlineStr">
@@ -9776,6 +10046,8 @@
       <c r="AZ126" s="59" t="n"/>
       <c r="BA126" s="59" t="n"/>
       <c r="BB126" s="59" t="n"/>
+      <c r="BC126" s="59" t="n"/>
+      <c r="BD126" s="59" t="n"/>
     </row>
     <row r="127" ht="13" customHeight="1">
       <c r="A127" s="60" t="n">
@@ -9791,10 +10063,10 @@
           <t>Ph.6</t>
         </is>
       </c>
-      <c r="D127" s="62" t="n">
+      <c r="D127" s="77" t="n">
         <v>46129</v>
       </c>
-      <c r="E127" s="62" t="n">
+      <c r="E127" s="77" t="n">
         <v>46130</v>
       </c>
       <c r="F127" s="60" t="n">
@@ -9848,6 +10120,8 @@
       <c r="AZ127" s="63" t="n"/>
       <c r="BA127" s="63" t="n"/>
       <c r="BB127" s="26" t="n"/>
+      <c r="BC127" s="26" t="n"/>
+      <c r="BD127" s="26" t="n"/>
     </row>
     <row r="128" ht="13" customHeight="1">
       <c r="A128" s="60" t="n">
@@ -9863,10 +10137,10 @@
           <t>Ph.6</t>
         </is>
       </c>
-      <c r="D128" s="62" t="n">
+      <c r="D128" s="77" t="n">
         <v>46129</v>
       </c>
-      <c r="E128" s="62" t="n">
+      <c r="E128" s="77" t="n">
         <v>46131</v>
       </c>
       <c r="F128" s="60" t="n">
@@ -9920,6 +10194,8 @@
       <c r="AZ128" s="63" t="n"/>
       <c r="BA128" s="63" t="n"/>
       <c r="BB128" s="26" t="n"/>
+      <c r="BC128" s="26" t="n"/>
+      <c r="BD128" s="26" t="n"/>
     </row>
     <row r="129" ht="13" customHeight="1">
       <c r="A129" s="60" t="n">
@@ -9935,10 +10211,10 @@
           <t>Ph.6</t>
         </is>
       </c>
-      <c r="D129" s="62" t="n">
+      <c r="D129" s="77" t="n">
         <v>46130</v>
       </c>
-      <c r="E129" s="62" t="n">
+      <c r="E129" s="77" t="n">
         <v>46131</v>
       </c>
       <c r="F129" s="60" t="n">
@@ -9992,6 +10268,8 @@
       <c r="AZ129" s="63" t="n"/>
       <c r="BA129" s="63" t="n"/>
       <c r="BB129" s="26" t="n"/>
+      <c r="BC129" s="26" t="n"/>
+      <c r="BD129" s="26" t="n"/>
     </row>
     <row r="130" ht="13" customHeight="1">
       <c r="A130" s="60" t="n">
@@ -10007,10 +10285,10 @@
           <t>Ph.6</t>
         </is>
       </c>
-      <c r="D130" s="62" t="n">
+      <c r="D130" s="77" t="n">
         <v>46131</v>
       </c>
-      <c r="E130" s="62" t="n">
+      <c r="E130" s="77" t="n">
         <v>46132</v>
       </c>
       <c r="F130" s="60" t="n">
@@ -10064,6 +10342,8 @@
       <c r="AZ130" s="63" t="n"/>
       <c r="BA130" s="63" t="n"/>
       <c r="BB130" s="26" t="n"/>
+      <c r="BC130" s="26" t="n"/>
+      <c r="BD130" s="26" t="n"/>
     </row>
     <row r="131" ht="13" customHeight="1">
       <c r="A131" s="60" t="n">
@@ -10079,10 +10359,10 @@
           <t>Ph.6</t>
         </is>
       </c>
-      <c r="D131" s="62" t="n">
+      <c r="D131" s="77" t="n">
         <v>46131</v>
       </c>
-      <c r="E131" s="62" t="n">
+      <c r="E131" s="77" t="n">
         <v>46132</v>
       </c>
       <c r="F131" s="60" t="n">
@@ -10136,6 +10416,8 @@
       <c r="AZ131" s="63" t="n"/>
       <c r="BA131" s="63" t="n"/>
       <c r="BB131" s="26" t="n"/>
+      <c r="BC131" s="26" t="n"/>
+      <c r="BD131" s="26" t="n"/>
     </row>
     <row r="132" ht="14" customHeight="1">
       <c r="A132" s="11" t="inlineStr">
@@ -10191,6 +10473,8 @@
       <c r="AZ132" s="65" t="n"/>
       <c r="BA132" s="65" t="n"/>
       <c r="BB132" s="65" t="n"/>
+      <c r="BC132" s="65" t="n"/>
+      <c r="BD132" s="65" t="n"/>
     </row>
     <row r="133" ht="13" customHeight="1">
       <c r="A133" s="66" t="n">
@@ -10206,10 +10490,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D133" s="68" t="n">
+      <c r="D133" s="78" t="n">
         <v>46129</v>
       </c>
-      <c r="E133" s="68" t="n">
+      <c r="E133" s="78" t="n">
         <v>46130</v>
       </c>
       <c r="F133" s="66" t="n">
@@ -10263,6 +10547,8 @@
       <c r="AZ133" s="69" t="n"/>
       <c r="BA133" s="69" t="n"/>
       <c r="BB133" s="26" t="n"/>
+      <c r="BC133" s="26" t="n"/>
+      <c r="BD133" s="26" t="n"/>
     </row>
     <row r="134" ht="13" customHeight="1">
       <c r="A134" s="66" t="n">
@@ -10278,10 +10564,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D134" s="68" t="n">
+      <c r="D134" s="78" t="n">
         <v>46129</v>
       </c>
-      <c r="E134" s="68" t="n">
+      <c r="E134" s="78" t="n">
         <v>46130</v>
       </c>
       <c r="F134" s="66" t="n">
@@ -10335,6 +10621,8 @@
       <c r="AZ134" s="69" t="n"/>
       <c r="BA134" s="69" t="n"/>
       <c r="BB134" s="26" t="n"/>
+      <c r="BC134" s="26" t="n"/>
+      <c r="BD134" s="26" t="n"/>
     </row>
     <row r="135" ht="13" customHeight="1">
       <c r="A135" s="66" t="n">
@@ -10350,10 +10638,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D135" s="68" t="n">
+      <c r="D135" s="78" t="n">
         <v>46129</v>
       </c>
-      <c r="E135" s="68" t="n">
+      <c r="E135" s="78" t="n">
         <v>46130</v>
       </c>
       <c r="F135" s="66" t="n">
@@ -10407,6 +10695,8 @@
       <c r="AZ135" s="69" t="n"/>
       <c r="BA135" s="69" t="n"/>
       <c r="BB135" s="26" t="n"/>
+      <c r="BC135" s="26" t="n"/>
+      <c r="BD135" s="26" t="n"/>
     </row>
     <row r="136" ht="13" customHeight="1">
       <c r="A136" s="66" t="n">
@@ -10422,10 +10712,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D136" s="68" t="n">
+      <c r="D136" s="78" t="n">
         <v>46130</v>
       </c>
-      <c r="E136" s="68" t="n">
+      <c r="E136" s="78" t="n">
         <v>46131</v>
       </c>
       <c r="F136" s="66" t="n">
@@ -10479,6 +10769,8 @@
       <c r="AZ136" s="69" t="n"/>
       <c r="BA136" s="69" t="n"/>
       <c r="BB136" s="26" t="n"/>
+      <c r="BC136" s="26" t="n"/>
+      <c r="BD136" s="26" t="n"/>
     </row>
     <row r="137" ht="13" customHeight="1">
       <c r="A137" s="66" t="n">
@@ -10494,10 +10786,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D137" s="68" t="n">
+      <c r="D137" s="78" t="n">
         <v>46130</v>
       </c>
-      <c r="E137" s="68" t="n">
+      <c r="E137" s="78" t="n">
         <v>46131</v>
       </c>
       <c r="F137" s="66" t="n">
@@ -10551,6 +10843,8 @@
       <c r="AZ137" s="69" t="n"/>
       <c r="BA137" s="69" t="n"/>
       <c r="BB137" s="26" t="n"/>
+      <c r="BC137" s="26" t="n"/>
+      <c r="BD137" s="26" t="n"/>
     </row>
     <row r="138" ht="13" customHeight="1">
       <c r="A138" s="66" t="n">
@@ -10566,10 +10860,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D138" s="68" t="n">
+      <c r="D138" s="78" t="n">
         <v>46130</v>
       </c>
-      <c r="E138" s="68" t="n">
+      <c r="E138" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F138" s="66" t="n">
@@ -10623,6 +10917,8 @@
       <c r="AZ138" s="69" t="n"/>
       <c r="BA138" s="69" t="n"/>
       <c r="BB138" s="26" t="n"/>
+      <c r="BC138" s="26" t="n"/>
+      <c r="BD138" s="26" t="n"/>
     </row>
     <row r="139" ht="13" customHeight="1">
       <c r="A139" s="66" t="n">
@@ -10638,10 +10934,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D139" s="68" t="n">
+      <c r="D139" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E139" s="68" t="n">
+      <c r="E139" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F139" s="66" t="n">
@@ -10695,6 +10991,8 @@
       <c r="AZ139" s="69" t="n"/>
       <c r="BA139" s="69" t="n"/>
       <c r="BB139" s="26" t="n"/>
+      <c r="BC139" s="26" t="n"/>
+      <c r="BD139" s="26" t="n"/>
     </row>
     <row r="140" ht="13" customHeight="1">
       <c r="A140" s="66" t="n">
@@ -10710,10 +11008,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D140" s="68" t="n">
+      <c r="D140" s="78" t="n">
         <v>46130</v>
       </c>
-      <c r="E140" s="68" t="n">
+      <c r="E140" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F140" s="66" t="n">
@@ -10767,6 +11065,8 @@
       <c r="AZ140" s="69" t="n"/>
       <c r="BA140" s="69" t="n"/>
       <c r="BB140" s="26" t="n"/>
+      <c r="BC140" s="26" t="n"/>
+      <c r="BD140" s="26" t="n"/>
     </row>
     <row r="141" ht="13" customHeight="1">
       <c r="A141" s="66" t="n">
@@ -10782,10 +11082,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D141" s="68" t="n">
+      <c r="D141" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E141" s="68" t="n">
+      <c r="E141" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F141" s="66" t="n">
@@ -10839,6 +11139,8 @@
       <c r="AZ141" s="69" t="n"/>
       <c r="BA141" s="69" t="n"/>
       <c r="BB141" s="26" t="n"/>
+      <c r="BC141" s="26" t="n"/>
+      <c r="BD141" s="26" t="n"/>
     </row>
     <row r="142" ht="13" customHeight="1">
       <c r="A142" s="66" t="n">
@@ -10854,10 +11156,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D142" s="68" t="n">
+      <c r="D142" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E142" s="68" t="n">
+      <c r="E142" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F142" s="66" t="n">
@@ -10911,6 +11213,8 @@
       <c r="AZ142" s="69" t="n"/>
       <c r="BA142" s="69" t="n"/>
       <c r="BB142" s="26" t="n"/>
+      <c r="BC142" s="26" t="n"/>
+      <c r="BD142" s="26" t="n"/>
     </row>
     <row r="143" ht="13" customHeight="1">
       <c r="A143" s="66" t="n">
@@ -10926,10 +11230,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D143" s="68" t="n">
+      <c r="D143" s="78" t="n">
         <v>46130</v>
       </c>
-      <c r="E143" s="68" t="n">
+      <c r="E143" s="78" t="n">
         <v>46131</v>
       </c>
       <c r="F143" s="66" t="n">
@@ -10983,6 +11287,8 @@
       <c r="AZ143" s="69" t="n"/>
       <c r="BA143" s="69" t="n"/>
       <c r="BB143" s="26" t="n"/>
+      <c r="BC143" s="26" t="n"/>
+      <c r="BD143" s="26" t="n"/>
     </row>
     <row r="144" ht="13" customHeight="1">
       <c r="A144" s="66" t="n">
@@ -10998,10 +11304,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D144" s="68" t="n">
+      <c r="D144" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E144" s="68" t="n">
+      <c r="E144" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F144" s="66" t="n">
@@ -11055,6 +11361,8 @@
       <c r="AZ144" s="69" t="n"/>
       <c r="BA144" s="69" t="n"/>
       <c r="BB144" s="26" t="n"/>
+      <c r="BC144" s="26" t="n"/>
+      <c r="BD144" s="26" t="n"/>
     </row>
     <row r="145" ht="13" customHeight="1">
       <c r="A145" s="66" t="n">
@@ -11070,10 +11378,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D145" s="68" t="n">
+      <c r="D145" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E145" s="68" t="n">
+      <c r="E145" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F145" s="66" t="n">
@@ -11127,6 +11435,8 @@
       <c r="AZ145" s="69" t="n"/>
       <c r="BA145" s="69" t="n"/>
       <c r="BB145" s="26" t="n"/>
+      <c r="BC145" s="26" t="n"/>
+      <c r="BD145" s="26" t="n"/>
     </row>
     <row r="146" ht="13" customHeight="1">
       <c r="A146" s="66" t="n">
@@ -11142,10 +11452,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D146" s="68" t="n">
+      <c r="D146" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E146" s="68" t="n">
+      <c r="E146" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F146" s="66" t="n">
@@ -11199,6 +11509,8 @@
       <c r="AZ146" s="69" t="n"/>
       <c r="BA146" s="69" t="n"/>
       <c r="BB146" s="26" t="n"/>
+      <c r="BC146" s="26" t="n"/>
+      <c r="BD146" s="26" t="n"/>
     </row>
     <row r="147" ht="13" customHeight="1">
       <c r="A147" s="66" t="n">
@@ -11214,10 +11526,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D147" s="68" t="n">
+      <c r="D147" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E147" s="68" t="n">
+      <c r="E147" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F147" s="66" t="n">
@@ -11275,6 +11587,8 @@
       <c r="AZ147" s="69" t="n"/>
       <c r="BA147" s="69" t="n"/>
       <c r="BB147" s="26" t="n"/>
+      <c r="BC147" s="26" t="n"/>
+      <c r="BD147" s="26" t="n"/>
     </row>
     <row r="148" ht="13" customHeight="1">
       <c r="A148" s="66" t="n">
@@ -11290,10 +11604,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D148" s="68" t="n">
+      <c r="D148" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E148" s="68" t="n">
+      <c r="E148" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F148" s="66" t="n">
@@ -11347,6 +11661,8 @@
       <c r="AZ148" s="69" t="n"/>
       <c r="BA148" s="69" t="n"/>
       <c r="BB148" s="26" t="n"/>
+      <c r="BC148" s="26" t="n"/>
+      <c r="BD148" s="26" t="n"/>
     </row>
     <row r="149" ht="13" customHeight="1">
       <c r="A149" s="66" t="n">
@@ -11362,10 +11678,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D149" s="68" t="n">
+      <c r="D149" s="78" t="n">
         <v>46131</v>
       </c>
-      <c r="E149" s="68" t="n">
+      <c r="E149" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F149" s="66" t="n">
@@ -11419,6 +11735,8 @@
       <c r="AZ149" s="69" t="n"/>
       <c r="BA149" s="69" t="n"/>
       <c r="BB149" s="26" t="n"/>
+      <c r="BC149" s="26" t="n"/>
+      <c r="BD149" s="26" t="n"/>
     </row>
     <row r="150" ht="13" customHeight="1">
       <c r="A150" s="66" t="n">
@@ -11434,10 +11752,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D150" s="68" t="n">
+      <c r="D150" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E150" s="68" t="n">
+      <c r="E150" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F150" s="66" t="n">
@@ -11491,6 +11809,8 @@
       <c r="AZ150" s="69" t="n"/>
       <c r="BA150" s="69" t="n"/>
       <c r="BB150" s="26" t="n"/>
+      <c r="BC150" s="26" t="n"/>
+      <c r="BD150" s="26" t="n"/>
     </row>
     <row r="151" ht="13" customHeight="1">
       <c r="A151" s="66" t="n">
@@ -11506,10 +11826,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D151" s="68" t="n">
+      <c r="D151" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E151" s="68" t="n">
+      <c r="E151" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F151" s="66" t="n">
@@ -11563,6 +11883,8 @@
       <c r="AZ151" s="69" t="n"/>
       <c r="BA151" s="69" t="n"/>
       <c r="BB151" s="26" t="n"/>
+      <c r="BC151" s="26" t="n"/>
+      <c r="BD151" s="26" t="n"/>
     </row>
     <row r="152" ht="13" customHeight="1">
       <c r="A152" s="66" t="n">
@@ -11578,10 +11900,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D152" s="68" t="n">
+      <c r="D152" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E152" s="68" t="n">
+      <c r="E152" s="78" t="n">
         <v>46132</v>
       </c>
       <c r="F152" s="66" t="n">
@@ -11639,6 +11961,8 @@
       <c r="AZ152" s="69" t="n"/>
       <c r="BA152" s="69" t="n"/>
       <c r="BB152" s="26" t="n"/>
+      <c r="BC152" s="26" t="n"/>
+      <c r="BD152" s="26" t="n"/>
     </row>
     <row r="153" ht="13" customHeight="1">
       <c r="A153" s="66" t="n">
@@ -11654,10 +11978,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D153" s="68" t="n">
+      <c r="D153" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E153" s="68" t="n">
+      <c r="E153" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F153" s="66" t="n">
@@ -11711,6 +12035,8 @@
       <c r="AZ153" s="69" t="n"/>
       <c r="BA153" s="69" t="n"/>
       <c r="BB153" s="26" t="n"/>
+      <c r="BC153" s="26" t="n"/>
+      <c r="BD153" s="26" t="n"/>
     </row>
     <row r="154" ht="13" customHeight="1">
       <c r="A154" s="66" t="n">
@@ -11726,10 +12052,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D154" s="68" t="n">
+      <c r="D154" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E154" s="68" t="n">
+      <c r="E154" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F154" s="66" t="n">
@@ -11783,6 +12109,8 @@
       <c r="AZ154" s="69" t="n"/>
       <c r="BA154" s="69" t="n"/>
       <c r="BB154" s="26" t="n"/>
+      <c r="BC154" s="26" t="n"/>
+      <c r="BD154" s="26" t="n"/>
     </row>
     <row r="155" ht="13" customHeight="1">
       <c r="A155" s="66" t="n">
@@ -11798,10 +12126,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D155" s="68" t="n">
+      <c r="D155" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E155" s="68" t="n">
+      <c r="E155" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F155" s="66" t="n">
@@ -11855,6 +12183,8 @@
       <c r="AZ155" s="69" t="n"/>
       <c r="BA155" s="69" t="n"/>
       <c r="BB155" s="26" t="n"/>
+      <c r="BC155" s="26" t="n"/>
+      <c r="BD155" s="26" t="n"/>
     </row>
     <row r="156" ht="13" customHeight="1">
       <c r="A156" s="66" t="n">
@@ -11870,10 +12200,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D156" s="68" t="n">
+      <c r="D156" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E156" s="68" t="n">
+      <c r="E156" s="78" t="n">
         <v>46134</v>
       </c>
       <c r="F156" s="66" t="n">
@@ -11927,6 +12257,8 @@
       <c r="AZ156" s="69" t="n"/>
       <c r="BA156" s="69" t="n"/>
       <c r="BB156" s="26" t="n"/>
+      <c r="BC156" s="26" t="n"/>
+      <c r="BD156" s="26" t="n"/>
     </row>
     <row r="157" ht="13" customHeight="1">
       <c r="A157" s="66" t="n">
@@ -11942,10 +12274,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D157" s="68" t="n">
+      <c r="D157" s="78" t="n">
         <v>46133</v>
       </c>
-      <c r="E157" s="68" t="n">
+      <c r="E157" s="78" t="n">
         <v>46134</v>
       </c>
       <c r="F157" s="66" t="n">
@@ -11999,6 +12331,8 @@
       <c r="AZ157" s="69" t="n"/>
       <c r="BA157" s="69" t="n"/>
       <c r="BB157" s="26" t="n"/>
+      <c r="BC157" s="26" t="n"/>
+      <c r="BD157" s="26" t="n"/>
     </row>
     <row r="158" ht="13" customHeight="1">
       <c r="A158" s="66" t="n">
@@ -12014,10 +12348,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D158" s="68" t="n">
+      <c r="D158" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E158" s="68" t="n">
+      <c r="E158" s="78" t="n">
         <v>46133</v>
       </c>
       <c r="F158" s="66" t="n">
@@ -12071,6 +12405,8 @@
       <c r="AZ158" s="69" t="n"/>
       <c r="BA158" s="69" t="n"/>
       <c r="BB158" s="26" t="n"/>
+      <c r="BC158" s="26" t="n"/>
+      <c r="BD158" s="26" t="n"/>
     </row>
     <row r="159" ht="13" customHeight="1">
       <c r="A159" s="66" t="n">
@@ -12086,10 +12422,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D159" s="68" t="n">
+      <c r="D159" s="78" t="n">
         <v>46133</v>
       </c>
-      <c r="E159" s="68" t="n">
+      <c r="E159" s="78" t="n">
         <v>46134</v>
       </c>
       <c r="F159" s="66" t="n">
@@ -12143,6 +12479,8 @@
       <c r="AZ159" s="69" t="n"/>
       <c r="BA159" s="69" t="n"/>
       <c r="BB159" s="26" t="n"/>
+      <c r="BC159" s="26" t="n"/>
+      <c r="BD159" s="26" t="n"/>
     </row>
     <row r="160" ht="13" customHeight="1">
       <c r="A160" s="66" t="n">
@@ -12158,10 +12496,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D160" s="68" t="n">
+      <c r="D160" s="78" t="n">
         <v>46132</v>
       </c>
-      <c r="E160" s="68" t="n">
+      <c r="E160" s="78" t="n">
         <v>46134</v>
       </c>
       <c r="F160" s="66" t="n">
@@ -12215,6 +12553,8 @@
       <c r="AZ160" s="69" t="n"/>
       <c r="BA160" s="69" t="n"/>
       <c r="BB160" s="26" t="n"/>
+      <c r="BC160" s="26" t="n"/>
+      <c r="BD160" s="26" t="n"/>
     </row>
     <row r="161" ht="13" customHeight="1">
       <c r="A161" s="66" t="n">
@@ -12230,10 +12570,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D161" s="68" t="n">
+      <c r="D161" s="78" t="n">
         <v>46134</v>
       </c>
-      <c r="E161" s="68" t="n">
+      <c r="E161" s="78" t="n">
         <v>46135</v>
       </c>
       <c r="F161" s="66" t="n">
@@ -12287,6 +12627,8 @@
       <c r="AZ161" s="70" t="n"/>
       <c r="BA161" s="69" t="n"/>
       <c r="BB161" s="26" t="n"/>
+      <c r="BC161" s="26" t="n"/>
+      <c r="BD161" s="26" t="n"/>
     </row>
     <row r="162" ht="13" customHeight="1">
       <c r="A162" s="66" t="n">
@@ -12302,10 +12644,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D162" s="68" t="n">
+      <c r="D162" s="78" t="n">
         <v>46134</v>
       </c>
-      <c r="E162" s="68" t="n">
+      <c r="E162" s="78" t="n">
         <v>46135</v>
       </c>
       <c r="F162" s="66" t="n">
@@ -12359,6 +12701,8 @@
       <c r="AZ162" s="70" t="n"/>
       <c r="BA162" s="69" t="n"/>
       <c r="BB162" s="26" t="n"/>
+      <c r="BC162" s="26" t="n"/>
+      <c r="BD162" s="26" t="n"/>
     </row>
     <row r="163" ht="13" customHeight="1">
       <c r="A163" s="66" t="n">
@@ -12374,10 +12718,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D163" s="68" t="n">
+      <c r="D163" s="78" t="n">
         <v>46133</v>
       </c>
-      <c r="E163" s="68" t="n">
+      <c r="E163" s="78" t="n">
         <v>46134</v>
       </c>
       <c r="F163" s="66" t="n">
@@ -12431,6 +12775,8 @@
       <c r="AZ163" s="69" t="n"/>
       <c r="BA163" s="69" t="n"/>
       <c r="BB163" s="26" t="n"/>
+      <c r="BC163" s="26" t="n"/>
+      <c r="BD163" s="26" t="n"/>
     </row>
     <row r="164" ht="13" customHeight="1">
       <c r="A164" s="66" t="n">
@@ -12446,10 +12792,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D164" s="68" t="n">
+      <c r="D164" s="78" t="n">
         <v>46134</v>
       </c>
-      <c r="E164" s="68" t="n">
+      <c r="E164" s="78" t="n">
         <v>46136</v>
       </c>
       <c r="F164" s="66" t="n">
@@ -12503,6 +12849,8 @@
       <c r="AZ164" s="70" t="n"/>
       <c r="BA164" s="70" t="n"/>
       <c r="BB164" s="26" t="n"/>
+      <c r="BC164" s="26" t="n"/>
+      <c r="BD164" s="26" t="n"/>
     </row>
     <row r="165" ht="13" customHeight="1">
       <c r="A165" s="66" t="n">
@@ -12518,10 +12866,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D165" s="68" t="n">
+      <c r="D165" s="78" t="n">
         <v>46135</v>
       </c>
-      <c r="E165" s="68" t="n">
+      <c r="E165" s="78" t="n">
         <v>46136</v>
       </c>
       <c r="F165" s="66" t="n">
@@ -12575,6 +12923,8 @@
       <c r="AZ165" s="70" t="n"/>
       <c r="BA165" s="70" t="n"/>
       <c r="BB165" s="26" t="n"/>
+      <c r="BC165" s="26" t="n"/>
+      <c r="BD165" s="26" t="n"/>
     </row>
     <row r="166" ht="13" customHeight="1">
       <c r="A166" s="66" t="n">
@@ -12590,10 +12940,10 @@
           <t>Ph.7</t>
         </is>
       </c>
-      <c r="D166" s="68" t="n">
+      <c r="D166" s="78" t="n">
         <v>46135</v>
       </c>
-      <c r="E166" s="68" t="n">
+      <c r="E166" s="78" t="n">
         <v>46137</v>
       </c>
       <c r="F166" s="66" t="n">
@@ -12647,15 +12997,703 @@
       <c r="AZ166" s="70" t="n"/>
       <c r="BA166" s="70" t="n"/>
       <c r="BB166" s="70" t="n"/>
+      <c r="BC166" s="70" t="n"/>
+      <c r="BD166" s="70" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▸  PHASE 8 — FINALISATION SOUTENANCE ET NETTOYAGE</t>
+        </is>
+      </c>
+      <c r="G167" s="65" t="n"/>
+      <c r="H167" s="65" t="n"/>
+      <c r="I167" s="65" t="n"/>
+      <c r="J167" s="65" t="n"/>
+      <c r="K167" s="65" t="n"/>
+      <c r="L167" s="65" t="n"/>
+      <c r="M167" s="65" t="n"/>
+      <c r="N167" s="65" t="n"/>
+      <c r="O167" s="65" t="n"/>
+      <c r="P167" s="65" t="n"/>
+      <c r="Q167" s="65" t="n"/>
+      <c r="R167" s="65" t="n"/>
+      <c r="S167" s="65" t="n"/>
+      <c r="T167" s="65" t="n"/>
+      <c r="U167" s="65" t="n"/>
+      <c r="V167" s="65" t="n"/>
+      <c r="W167" s="65" t="n"/>
+      <c r="X167" s="65" t="n"/>
+      <c r="Y167" s="65" t="n"/>
+      <c r="Z167" s="65" t="n"/>
+      <c r="AA167" s="65" t="n"/>
+      <c r="AB167" s="65" t="n"/>
+      <c r="AC167" s="65" t="n"/>
+      <c r="AD167" s="65" t="n"/>
+      <c r="AE167" s="65" t="n"/>
+      <c r="AF167" s="65" t="n"/>
+      <c r="AG167" s="65" t="n"/>
+      <c r="AH167" s="65" t="n"/>
+      <c r="AI167" s="65" t="n"/>
+      <c r="AJ167" s="65" t="n"/>
+      <c r="AK167" s="65" t="n"/>
+      <c r="AL167" s="65" t="n"/>
+      <c r="AM167" s="65" t="n"/>
+      <c r="AN167" s="65" t="n"/>
+      <c r="AO167" s="65" t="n"/>
+      <c r="AP167" s="65" t="n"/>
+      <c r="AQ167" s="65" t="n"/>
+      <c r="AR167" s="65" t="n"/>
+      <c r="AS167" s="65" t="n"/>
+      <c r="AT167" s="65" t="n"/>
+      <c r="AU167" s="65" t="n"/>
+      <c r="AV167" s="65" t="n"/>
+      <c r="AW167" s="65" t="n"/>
+      <c r="AX167" s="65" t="n"/>
+      <c r="AY167" s="65" t="n"/>
+      <c r="AZ167" s="65" t="n"/>
+      <c r="BA167" s="65" t="n"/>
+      <c r="BB167" s="65" t="n"/>
+      <c r="BC167" s="65" t="n"/>
+      <c r="BD167" s="65" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="66" t="n">
+        <v>150</v>
+      </c>
+      <c r="B168" s="67" t="inlineStr">
+        <is>
+          <t>Séparation headers/implémentations (.h → .cpp)</t>
+        </is>
+      </c>
+      <c r="C168" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D168" s="78" t="n">
+        <v>46138</v>
+      </c>
+      <c r="E168" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F168" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="G168" s="69" t="n"/>
+      <c r="H168" s="69" t="n"/>
+      <c r="I168" s="69" t="n"/>
+      <c r="J168" s="69" t="n"/>
+      <c r="K168" s="69" t="n"/>
+      <c r="L168" s="26" t="n"/>
+      <c r="M168" s="26" t="n"/>
+      <c r="N168" s="69" t="n"/>
+      <c r="O168" s="69" t="n"/>
+      <c r="P168" s="69" t="n"/>
+      <c r="Q168" s="69" t="n"/>
+      <c r="R168" s="69" t="n"/>
+      <c r="S168" s="26" t="n"/>
+      <c r="T168" s="26" t="n"/>
+      <c r="U168" s="69" t="n"/>
+      <c r="V168" s="69" t="n"/>
+      <c r="W168" s="69" t="n"/>
+      <c r="X168" s="69" t="n"/>
+      <c r="Y168" s="69" t="n"/>
+      <c r="Z168" s="26" t="n"/>
+      <c r="AA168" s="26" t="n"/>
+      <c r="AB168" s="69" t="n"/>
+      <c r="AC168" s="69" t="n"/>
+      <c r="AD168" s="69" t="n"/>
+      <c r="AE168" s="69" t="n"/>
+      <c r="AF168" s="69" t="n"/>
+      <c r="AG168" s="26" t="n"/>
+      <c r="AH168" s="26" t="n"/>
+      <c r="AI168" s="69" t="n"/>
+      <c r="AJ168" s="69" t="n"/>
+      <c r="AK168" s="69" t="n"/>
+      <c r="AL168" s="69" t="n"/>
+      <c r="AM168" s="69" t="n"/>
+      <c r="AN168" s="26" t="n"/>
+      <c r="AO168" s="26" t="n"/>
+      <c r="AP168" s="69" t="n"/>
+      <c r="AQ168" s="69" t="n"/>
+      <c r="AR168" s="69" t="n"/>
+      <c r="AS168" s="69" t="n"/>
+      <c r="AT168" s="69" t="n"/>
+      <c r="AU168" s="26" t="n"/>
+      <c r="AV168" s="26" t="n"/>
+      <c r="AW168" s="69" t="n"/>
+      <c r="AX168" s="69" t="n"/>
+      <c r="AY168" s="69" t="n"/>
+      <c r="AZ168" s="70" t="n"/>
+      <c r="BA168" s="70" t="n"/>
+      <c r="BB168" s="70" t="n"/>
+      <c r="BC168" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="BD168" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="66" t="n">
+        <v>151</v>
+      </c>
+      <c r="B169" s="67" t="inlineStr">
+        <is>
+          <t>Passage paramètres non triviaux en const&amp;</t>
+        </is>
+      </c>
+      <c r="C169" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D169" s="78" t="n">
+        <v>46138</v>
+      </c>
+      <c r="E169" s="78" t="n">
+        <v>46138</v>
+      </c>
+      <c r="F169" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G169" s="69" t="n"/>
+      <c r="H169" s="69" t="n"/>
+      <c r="I169" s="69" t="n"/>
+      <c r="J169" s="69" t="n"/>
+      <c r="K169" s="69" t="n"/>
+      <c r="L169" s="26" t="n"/>
+      <c r="M169" s="26" t="n"/>
+      <c r="N169" s="69" t="n"/>
+      <c r="O169" s="69" t="n"/>
+      <c r="P169" s="69" t="n"/>
+      <c r="Q169" s="69" t="n"/>
+      <c r="R169" s="69" t="n"/>
+      <c r="S169" s="26" t="n"/>
+      <c r="T169" s="26" t="n"/>
+      <c r="U169" s="69" t="n"/>
+      <c r="V169" s="69" t="n"/>
+      <c r="W169" s="69" t="n"/>
+      <c r="X169" s="69" t="n"/>
+      <c r="Y169" s="69" t="n"/>
+      <c r="Z169" s="26" t="n"/>
+      <c r="AA169" s="26" t="n"/>
+      <c r="AB169" s="69" t="n"/>
+      <c r="AC169" s="69" t="n"/>
+      <c r="AD169" s="69" t="n"/>
+      <c r="AE169" s="69" t="n"/>
+      <c r="AF169" s="69" t="n"/>
+      <c r="AG169" s="26" t="n"/>
+      <c r="AH169" s="26" t="n"/>
+      <c r="AI169" s="69" t="n"/>
+      <c r="AJ169" s="69" t="n"/>
+      <c r="AK169" s="69" t="n"/>
+      <c r="AL169" s="69" t="n"/>
+      <c r="AM169" s="69" t="n"/>
+      <c r="AN169" s="26" t="n"/>
+      <c r="AO169" s="26" t="n"/>
+      <c r="AP169" s="69" t="n"/>
+      <c r="AQ169" s="69" t="n"/>
+      <c r="AR169" s="69" t="n"/>
+      <c r="AS169" s="69" t="n"/>
+      <c r="AT169" s="69" t="n"/>
+      <c r="AU169" s="26" t="n"/>
+      <c r="AV169" s="26" t="n"/>
+      <c r="AW169" s="69" t="n"/>
+      <c r="AX169" s="69" t="n"/>
+      <c r="AY169" s="69" t="n"/>
+      <c r="AZ169" s="70" t="n"/>
+      <c r="BA169" s="70" t="n"/>
+      <c r="BB169" s="70" t="n"/>
+      <c r="BC169" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="BD169" s="70" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="66" t="n">
+        <v>152</v>
+      </c>
+      <c r="B170" s="67" t="inlineStr">
+        <is>
+          <t>Mise à jour Makefile pour les nouveaux .cpp</t>
+        </is>
+      </c>
+      <c r="C170" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D170" s="78" t="n">
+        <v>46138</v>
+      </c>
+      <c r="E170" s="78" t="n">
+        <v>46138</v>
+      </c>
+      <c r="F170" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G170" s="69" t="n"/>
+      <c r="H170" s="69" t="n"/>
+      <c r="I170" s="69" t="n"/>
+      <c r="J170" s="69" t="n"/>
+      <c r="K170" s="69" t="n"/>
+      <c r="L170" s="26" t="n"/>
+      <c r="M170" s="26" t="n"/>
+      <c r="N170" s="69" t="n"/>
+      <c r="O170" s="69" t="n"/>
+      <c r="P170" s="69" t="n"/>
+      <c r="Q170" s="69" t="n"/>
+      <c r="R170" s="69" t="n"/>
+      <c r="S170" s="26" t="n"/>
+      <c r="T170" s="26" t="n"/>
+      <c r="U170" s="69" t="n"/>
+      <c r="V170" s="69" t="n"/>
+      <c r="W170" s="69" t="n"/>
+      <c r="X170" s="69" t="n"/>
+      <c r="Y170" s="69" t="n"/>
+      <c r="Z170" s="26" t="n"/>
+      <c r="AA170" s="26" t="n"/>
+      <c r="AB170" s="69" t="n"/>
+      <c r="AC170" s="69" t="n"/>
+      <c r="AD170" s="69" t="n"/>
+      <c r="AE170" s="69" t="n"/>
+      <c r="AF170" s="69" t="n"/>
+      <c r="AG170" s="26" t="n"/>
+      <c r="AH170" s="26" t="n"/>
+      <c r="AI170" s="69" t="n"/>
+      <c r="AJ170" s="69" t="n"/>
+      <c r="AK170" s="69" t="n"/>
+      <c r="AL170" s="69" t="n"/>
+      <c r="AM170" s="69" t="n"/>
+      <c r="AN170" s="26" t="n"/>
+      <c r="AO170" s="26" t="n"/>
+      <c r="AP170" s="69" t="n"/>
+      <c r="AQ170" s="69" t="n"/>
+      <c r="AR170" s="69" t="n"/>
+      <c r="AS170" s="69" t="n"/>
+      <c r="AT170" s="69" t="n"/>
+      <c r="AU170" s="26" t="n"/>
+      <c r="AV170" s="26" t="n"/>
+      <c r="AW170" s="69" t="n"/>
+      <c r="AX170" s="69" t="n"/>
+      <c r="AY170" s="69" t="n"/>
+      <c r="AZ170" s="70" t="n"/>
+      <c r="BA170" s="70" t="n"/>
+      <c r="BB170" s="70" t="n"/>
+      <c r="BC170" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="BD170" s="70" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="66" t="n">
+        <v>153</v>
+      </c>
+      <c r="B171" s="67" t="inlineStr">
+        <is>
+          <t>Documentation pédagogique explication/</t>
+        </is>
+      </c>
+      <c r="C171" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D171" s="78" t="n">
+        <v>46137</v>
+      </c>
+      <c r="E171" s="78" t="n">
+        <v>46138</v>
+      </c>
+      <c r="F171" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="G171" s="69" t="n"/>
+      <c r="H171" s="69" t="n"/>
+      <c r="I171" s="69" t="n"/>
+      <c r="J171" s="69" t="n"/>
+      <c r="K171" s="69" t="n"/>
+      <c r="L171" s="26" t="n"/>
+      <c r="M171" s="26" t="n"/>
+      <c r="N171" s="69" t="n"/>
+      <c r="O171" s="69" t="n"/>
+      <c r="P171" s="69" t="n"/>
+      <c r="Q171" s="69" t="n"/>
+      <c r="R171" s="69" t="n"/>
+      <c r="S171" s="26" t="n"/>
+      <c r="T171" s="26" t="n"/>
+      <c r="U171" s="69" t="n"/>
+      <c r="V171" s="69" t="n"/>
+      <c r="W171" s="69" t="n"/>
+      <c r="X171" s="69" t="n"/>
+      <c r="Y171" s="69" t="n"/>
+      <c r="Z171" s="26" t="n"/>
+      <c r="AA171" s="26" t="n"/>
+      <c r="AB171" s="69" t="n"/>
+      <c r="AC171" s="69" t="n"/>
+      <c r="AD171" s="69" t="n"/>
+      <c r="AE171" s="69" t="n"/>
+      <c r="AF171" s="69" t="n"/>
+      <c r="AG171" s="26" t="n"/>
+      <c r="AH171" s="26" t="n"/>
+      <c r="AI171" s="69" t="n"/>
+      <c r="AJ171" s="69" t="n"/>
+      <c r="AK171" s="69" t="n"/>
+      <c r="AL171" s="69" t="n"/>
+      <c r="AM171" s="69" t="n"/>
+      <c r="AN171" s="26" t="n"/>
+      <c r="AO171" s="26" t="n"/>
+      <c r="AP171" s="69" t="n"/>
+      <c r="AQ171" s="69" t="n"/>
+      <c r="AR171" s="69" t="n"/>
+      <c r="AS171" s="69" t="n"/>
+      <c r="AT171" s="69" t="n"/>
+      <c r="AU171" s="26" t="n"/>
+      <c r="AV171" s="26" t="n"/>
+      <c r="AW171" s="69" t="n"/>
+      <c r="AX171" s="69" t="n"/>
+      <c r="AY171" s="69" t="n"/>
+      <c r="AZ171" s="70" t="n"/>
+      <c r="BA171" s="70" t="n"/>
+      <c r="BB171" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="BC171" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="BD171" s="70" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="66" t="n">
+        <v>154</v>
+      </c>
+      <c r="B172" s="67" t="inlineStr">
+        <is>
+          <t>Réorganisation assets présentation images/videos/diagrams/notes</t>
+        </is>
+      </c>
+      <c r="C172" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D172" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E172" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F172" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G172" s="69" t="n"/>
+      <c r="H172" s="69" t="n"/>
+      <c r="I172" s="69" t="n"/>
+      <c r="J172" s="69" t="n"/>
+      <c r="K172" s="69" t="n"/>
+      <c r="L172" s="26" t="n"/>
+      <c r="M172" s="26" t="n"/>
+      <c r="N172" s="69" t="n"/>
+      <c r="O172" s="69" t="n"/>
+      <c r="P172" s="69" t="n"/>
+      <c r="Q172" s="69" t="n"/>
+      <c r="R172" s="69" t="n"/>
+      <c r="S172" s="26" t="n"/>
+      <c r="T172" s="26" t="n"/>
+      <c r="U172" s="69" t="n"/>
+      <c r="V172" s="69" t="n"/>
+      <c r="W172" s="69" t="n"/>
+      <c r="X172" s="69" t="n"/>
+      <c r="Y172" s="69" t="n"/>
+      <c r="Z172" s="26" t="n"/>
+      <c r="AA172" s="26" t="n"/>
+      <c r="AB172" s="69" t="n"/>
+      <c r="AC172" s="69" t="n"/>
+      <c r="AD172" s="69" t="n"/>
+      <c r="AE172" s="69" t="n"/>
+      <c r="AF172" s="69" t="n"/>
+      <c r="AG172" s="26" t="n"/>
+      <c r="AH172" s="26" t="n"/>
+      <c r="AI172" s="69" t="n"/>
+      <c r="AJ172" s="69" t="n"/>
+      <c r="AK172" s="69" t="n"/>
+      <c r="AL172" s="69" t="n"/>
+      <c r="AM172" s="69" t="n"/>
+      <c r="AN172" s="26" t="n"/>
+      <c r="AO172" s="26" t="n"/>
+      <c r="AP172" s="69" t="n"/>
+      <c r="AQ172" s="69" t="n"/>
+      <c r="AR172" s="69" t="n"/>
+      <c r="AS172" s="69" t="n"/>
+      <c r="AT172" s="69" t="n"/>
+      <c r="AU172" s="26" t="n"/>
+      <c r="AV172" s="26" t="n"/>
+      <c r="AW172" s="69" t="n"/>
+      <c r="AX172" s="69" t="n"/>
+      <c r="AY172" s="69" t="n"/>
+      <c r="AZ172" s="70" t="n"/>
+      <c r="BA172" s="70" t="n"/>
+      <c r="BB172" s="70" t="n"/>
+      <c r="BC172" s="70" t="n"/>
+      <c r="BD172" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="66" t="n">
+        <v>155</v>
+      </c>
+      <c r="B173" s="67" t="inlineStr">
+        <is>
+          <t>Nettoyage doc/presentation — conservation presentation_shell.html</t>
+        </is>
+      </c>
+      <c r="C173" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D173" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E173" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F173" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G173" s="69" t="n"/>
+      <c r="H173" s="69" t="n"/>
+      <c r="I173" s="69" t="n"/>
+      <c r="J173" s="69" t="n"/>
+      <c r="K173" s="69" t="n"/>
+      <c r="L173" s="26" t="n"/>
+      <c r="M173" s="26" t="n"/>
+      <c r="N173" s="69" t="n"/>
+      <c r="O173" s="69" t="n"/>
+      <c r="P173" s="69" t="n"/>
+      <c r="Q173" s="69" t="n"/>
+      <c r="R173" s="69" t="n"/>
+      <c r="S173" s="26" t="n"/>
+      <c r="T173" s="26" t="n"/>
+      <c r="U173" s="69" t="n"/>
+      <c r="V173" s="69" t="n"/>
+      <c r="W173" s="69" t="n"/>
+      <c r="X173" s="69" t="n"/>
+      <c r="Y173" s="69" t="n"/>
+      <c r="Z173" s="26" t="n"/>
+      <c r="AA173" s="26" t="n"/>
+      <c r="AB173" s="69" t="n"/>
+      <c r="AC173" s="69" t="n"/>
+      <c r="AD173" s="69" t="n"/>
+      <c r="AE173" s="69" t="n"/>
+      <c r="AF173" s="69" t="n"/>
+      <c r="AG173" s="26" t="n"/>
+      <c r="AH173" s="26" t="n"/>
+      <c r="AI173" s="69" t="n"/>
+      <c r="AJ173" s="69" t="n"/>
+      <c r="AK173" s="69" t="n"/>
+      <c r="AL173" s="69" t="n"/>
+      <c r="AM173" s="69" t="n"/>
+      <c r="AN173" s="26" t="n"/>
+      <c r="AO173" s="26" t="n"/>
+      <c r="AP173" s="69" t="n"/>
+      <c r="AQ173" s="69" t="n"/>
+      <c r="AR173" s="69" t="n"/>
+      <c r="AS173" s="69" t="n"/>
+      <c r="AT173" s="69" t="n"/>
+      <c r="AU173" s="26" t="n"/>
+      <c r="AV173" s="26" t="n"/>
+      <c r="AW173" s="69" t="n"/>
+      <c r="AX173" s="69" t="n"/>
+      <c r="AY173" s="69" t="n"/>
+      <c r="AZ173" s="70" t="n"/>
+      <c r="BA173" s="70" t="n"/>
+      <c r="BB173" s="70" t="n"/>
+      <c r="BC173" s="70" t="n"/>
+      <c r="BD173" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="66" t="n">
+        <v>156</v>
+      </c>
+      <c r="B174" s="67" t="inlineStr">
+        <is>
+          <t>Mise à jour class_diagram.md avec core/physics</t>
+        </is>
+      </c>
+      <c r="C174" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D174" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E174" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F174" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G174" s="69" t="n"/>
+      <c r="H174" s="69" t="n"/>
+      <c r="I174" s="69" t="n"/>
+      <c r="J174" s="69" t="n"/>
+      <c r="K174" s="69" t="n"/>
+      <c r="L174" s="26" t="n"/>
+      <c r="M174" s="26" t="n"/>
+      <c r="N174" s="69" t="n"/>
+      <c r="O174" s="69" t="n"/>
+      <c r="P174" s="69" t="n"/>
+      <c r="Q174" s="69" t="n"/>
+      <c r="R174" s="69" t="n"/>
+      <c r="S174" s="26" t="n"/>
+      <c r="T174" s="26" t="n"/>
+      <c r="U174" s="69" t="n"/>
+      <c r="V174" s="69" t="n"/>
+      <c r="W174" s="69" t="n"/>
+      <c r="X174" s="69" t="n"/>
+      <c r="Y174" s="69" t="n"/>
+      <c r="Z174" s="26" t="n"/>
+      <c r="AA174" s="26" t="n"/>
+      <c r="AB174" s="69" t="n"/>
+      <c r="AC174" s="69" t="n"/>
+      <c r="AD174" s="69" t="n"/>
+      <c r="AE174" s="69" t="n"/>
+      <c r="AF174" s="69" t="n"/>
+      <c r="AG174" s="26" t="n"/>
+      <c r="AH174" s="26" t="n"/>
+      <c r="AI174" s="69" t="n"/>
+      <c r="AJ174" s="69" t="n"/>
+      <c r="AK174" s="69" t="n"/>
+      <c r="AL174" s="69" t="n"/>
+      <c r="AM174" s="69" t="n"/>
+      <c r="AN174" s="26" t="n"/>
+      <c r="AO174" s="26" t="n"/>
+      <c r="AP174" s="69" t="n"/>
+      <c r="AQ174" s="69" t="n"/>
+      <c r="AR174" s="69" t="n"/>
+      <c r="AS174" s="69" t="n"/>
+      <c r="AT174" s="69" t="n"/>
+      <c r="AU174" s="26" t="n"/>
+      <c r="AV174" s="26" t="n"/>
+      <c r="AW174" s="69" t="n"/>
+      <c r="AX174" s="69" t="n"/>
+      <c r="AY174" s="69" t="n"/>
+      <c r="AZ174" s="70" t="n"/>
+      <c r="BA174" s="70" t="n"/>
+      <c r="BB174" s="70" t="n"/>
+      <c r="BC174" s="70" t="n"/>
+      <c r="BD174" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="66" t="n">
+        <v>157</v>
+      </c>
+      <c r="B175" s="67" t="inlineStr">
+        <is>
+          <t>Mise à jour finale du Gantt</t>
+        </is>
+      </c>
+      <c r="C175" s="66" t="inlineStr">
+        <is>
+          <t>Ph.8</t>
+        </is>
+      </c>
+      <c r="D175" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E175" s="78" t="n">
+        <v>46139</v>
+      </c>
+      <c r="F175" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G175" s="69" t="n"/>
+      <c r="H175" s="69" t="n"/>
+      <c r="I175" s="69" t="n"/>
+      <c r="J175" s="69" t="n"/>
+      <c r="K175" s="69" t="n"/>
+      <c r="L175" s="26" t="n"/>
+      <c r="M175" s="26" t="n"/>
+      <c r="N175" s="69" t="n"/>
+      <c r="O175" s="69" t="n"/>
+      <c r="P175" s="69" t="n"/>
+      <c r="Q175" s="69" t="n"/>
+      <c r="R175" s="69" t="n"/>
+      <c r="S175" s="26" t="n"/>
+      <c r="T175" s="26" t="n"/>
+      <c r="U175" s="69" t="n"/>
+      <c r="V175" s="69" t="n"/>
+      <c r="W175" s="69" t="n"/>
+      <c r="X175" s="69" t="n"/>
+      <c r="Y175" s="69" t="n"/>
+      <c r="Z175" s="26" t="n"/>
+      <c r="AA175" s="26" t="n"/>
+      <c r="AB175" s="69" t="n"/>
+      <c r="AC175" s="69" t="n"/>
+      <c r="AD175" s="69" t="n"/>
+      <c r="AE175" s="69" t="n"/>
+      <c r="AF175" s="69" t="n"/>
+      <c r="AG175" s="26" t="n"/>
+      <c r="AH175" s="26" t="n"/>
+      <c r="AI175" s="69" t="n"/>
+      <c r="AJ175" s="69" t="n"/>
+      <c r="AK175" s="69" t="n"/>
+      <c r="AL175" s="69" t="n"/>
+      <c r="AM175" s="69" t="n"/>
+      <c r="AN175" s="26" t="n"/>
+      <c r="AO175" s="26" t="n"/>
+      <c r="AP175" s="69" t="n"/>
+      <c r="AQ175" s="69" t="n"/>
+      <c r="AR175" s="69" t="n"/>
+      <c r="AS175" s="69" t="n"/>
+      <c r="AT175" s="69" t="n"/>
+      <c r="AU175" s="26" t="n"/>
+      <c r="AV175" s="26" t="n"/>
+      <c r="AW175" s="69" t="n"/>
+      <c r="AX175" s="69" t="n"/>
+      <c r="AY175" s="69" t="n"/>
+      <c r="AZ175" s="70" t="n"/>
+      <c r="BA175" s="70" t="n"/>
+      <c r="BB175" s="70" t="n"/>
+      <c r="BC175" s="70" t="n"/>
+      <c r="BD175" s="70" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="29">
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="AN4:BB4"/>
-    <mergeCell ref="A1:BB1"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A6:BB6"/>
-    <mergeCell ref="AD7:BB7"/>
     <mergeCell ref="C7:C9"/>
     <mergeCell ref="E7:E9"/>
     <mergeCell ref="A116:F116"/>
@@ -12663,18 +13701,22 @@
     <mergeCell ref="A106:F106"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="N4:Z4"/>
-    <mergeCell ref="A3:BB3"/>
     <mergeCell ref="G7:AC7"/>
+    <mergeCell ref="A1:BD1"/>
+    <mergeCell ref="A6:BD6"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A2:BB2"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="F7:F9"/>
+    <mergeCell ref="AD7:BD7"/>
+    <mergeCell ref="A167:F167"/>
     <mergeCell ref="AA5:AM5"/>
     <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A3:BD3"/>
     <mergeCell ref="N5:Z5"/>
     <mergeCell ref="A132:F132"/>
     <mergeCell ref="A79:F79"/>
+    <mergeCell ref="A2:BD2"/>
     <mergeCell ref="D7:D9"/>
     <mergeCell ref="AA4:AM4"/>
     <mergeCell ref="AN5:BB5"/>

</xml_diff>